<commit_message>
Need To rerun with correct F1
</commit_message>
<xml_diff>
--- a/Fit Results/AllFitsF1=4.xlsx
+++ b/Fit Results/AllFitsF1=4.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Diego\git\6s7p\Fit Results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9689E346-71C4-448B-B7D6-BFE2F6FAAC94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AF14773-0C0C-422C-BB11-EE17912AEF92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="All" sheetId="5" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="240">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="290">
   <si>
     <t>May22,2026+11-50-22AM</t>
   </si>
@@ -759,6 +759,156 @@
   </si>
   <si>
     <t>Jul09,2026+4-10-46PM</t>
+  </si>
+  <si>
+    <t>Jul13,2026+10-12-06AM</t>
+  </si>
+  <si>
+    <t>Jul13,2026+10-34-59AM</t>
+  </si>
+  <si>
+    <t>Jul13,2026+10-54-06AM</t>
+  </si>
+  <si>
+    <t>Jul13,2026+11-11-20AM</t>
+  </si>
+  <si>
+    <t>Jul13,2026+11-19-18AM</t>
+  </si>
+  <si>
+    <t>Jul13,2026+11-27-51AM</t>
+  </si>
+  <si>
+    <t>Jul13,2026+11-39-03AM</t>
+  </si>
+  <si>
+    <t>Jul13,2026+12-12-01PM</t>
+  </si>
+  <si>
+    <t>Jul13,2026+12-21-13PM</t>
+  </si>
+  <si>
+    <t>Jul13,2026+12-29-13PM</t>
+  </si>
+  <si>
+    <t>Jul13,2026+12-38-19PM</t>
+  </si>
+  <si>
+    <t>Jul13,2026+12-58-04PM</t>
+  </si>
+  <si>
+    <t>Jul13,2026+1-07-47PM</t>
+  </si>
+  <si>
+    <t>Jul13,2026+1-21-29PM</t>
+  </si>
+  <si>
+    <t>Jul13,2026+1-34-28PM</t>
+  </si>
+  <si>
+    <t>Jul13,2026+1-42-33PM</t>
+  </si>
+  <si>
+    <t>Jul13,2026+1-52-37PM</t>
+  </si>
+  <si>
+    <t>Jul13,2026+2-05-19PM</t>
+  </si>
+  <si>
+    <t>Jul13,2026+2-17-27PM</t>
+  </si>
+  <si>
+    <t>Jul13,2026+2-55-51PM</t>
+  </si>
+  <si>
+    <t>Jul13,2026+3-41-08PM</t>
+  </si>
+  <si>
+    <t>Jul13,2026+3-52-31PM</t>
+  </si>
+  <si>
+    <t>Jul13,2026+4-02-38PM</t>
+  </si>
+  <si>
+    <t>Jul13,2026+4-10-40PM</t>
+  </si>
+  <si>
+    <t>Jul13,2026+4-42-25PM</t>
+  </si>
+  <si>
+    <t>Jul13,2026+5-21-33PM</t>
+  </si>
+  <si>
+    <t>Jul13,2026+5-31-01PM</t>
+  </si>
+  <si>
+    <t>Jul13,2026+5-39-08PM</t>
+  </si>
+  <si>
+    <t>Jul14,2026+12-14-44PM</t>
+  </si>
+  <si>
+    <t>Jul14,2026+12-26-20PM</t>
+  </si>
+  <si>
+    <t>Jul14,2026+12-34-37PM</t>
+  </si>
+  <si>
+    <t>Jul14,2026+12-45-58PM</t>
+  </si>
+  <si>
+    <t>Jul14,2026+12-55-14PM</t>
+  </si>
+  <si>
+    <t>Jul14,2026+2-38-28PM</t>
+  </si>
+  <si>
+    <t>Jul14,2026+2-48-47PM</t>
+  </si>
+  <si>
+    <t>Jul14,2026+2-57-45PM</t>
+  </si>
+  <si>
+    <t>Jul14,2026+3-05-52PM</t>
+  </si>
+  <si>
+    <t>Jul14,2026+3-18-29PM</t>
+  </si>
+  <si>
+    <t>Jul14,2026+3-41-29PM</t>
+  </si>
+  <si>
+    <t>Jul14,2026+4-11-34PM</t>
+  </si>
+  <si>
+    <t>Jul14,2026+4-20-19PM</t>
+  </si>
+  <si>
+    <t>Jul14,2026+4-29-37PM</t>
+  </si>
+  <si>
+    <t>Jul14,2026+5-02-47PM</t>
+  </si>
+  <si>
+    <t>Jul14,2026+5-11-12PM</t>
+  </si>
+  <si>
+    <t>Jul14,2026+5-24-44PM</t>
+  </si>
+  <si>
+    <t>Jul14,2026+5-32-49PM</t>
+  </si>
+  <si>
+    <t>Jul14,2026+5-40-48PM</t>
+  </si>
+  <si>
+    <t>Jul14,2026+5-56-32PM</t>
+  </si>
+  <si>
+    <t>Jul14,2026+6-06-06PM</t>
+  </si>
+  <si>
+    <t>Jul14,2026+6-16-24PM</t>
   </si>
 </sst>
 </file>
@@ -2747,6 +2897,420 @@
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000002-A036-4546-BBC9-4080821F7EE7}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="10"/>
+          <c:order val="10"/>
+          <c:tx>
+            <c:v>13-Jul</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent5">
+                  <a:lumMod val="60000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent5">
+                    <a:lumMod val="60000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>All!$B$229:$B$256</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="28"/>
+                <c:pt idx="0">
+                  <c:v>4.0279639492061596</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>4.0667523488381301</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>4.0183878243548996</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4.0314213938624102</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>4.0505545969773804</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>4.0517862191438496</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>4.0424645012040497</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>4.0243487276243002</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>4.0367409025359304</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>4.0491156124478902</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>4.0406778045491096</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>4.0437611760653196</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>4.0356877834891698</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>4.0543291932026699</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>4.0440448461837999</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>4.0482658159189198</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>4.0372658698111801</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>4.0430873829414802</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>4.0311378792119203</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>4.01331392262989</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>4.0578910745577002</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>4.02794326730218</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>4.0616651770599299</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>4.02065487780051</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>4.0194143809069702</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>4.0195181922825496</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>4.0060394450385299</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>4.03113906858741</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>All!$C$229:$C$256</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="28"/>
+                <c:pt idx="0">
+                  <c:v>8.3409466599106696E-2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>8.3177485471750606E-2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>8.3006037660706203E-2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>8.3019038948826299E-2</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>8.3723462750931996E-2</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>8.3608574512507694E-2</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>8.3118939745191397E-2</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>8.3605447355610901E-2</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>8.3418150740260003E-2</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>8.3455841721042895E-2</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>8.3276939213918696E-2</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>8.3116670967641595E-2</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>8.3363484131550397E-2</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>8.3757021233168596E-2</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>8.3417811249936594E-2</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>8.4025870340482506E-2</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>8.2022959476588206E-2</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>8.3225256404970693E-2</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>8.2797901589345094E-2</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>8.4124029452458504E-2</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>8.2524964266572395E-2</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>8.3779837646985295E-2</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>8.2884597799815607E-2</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>8.3056026546302203E-2</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>8.3119909910801301E-2</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>8.29152163470048E-2</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>8.28084692004942E-2</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>8.3334028420614895E-2</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-0A5E-41D6-B680-57131B471AE9}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="11"/>
+          <c:order val="11"/>
+          <c:tx>
+            <c:v>14-Jul</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent6">
+                  <a:lumMod val="60000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent6">
+                    <a:lumMod val="60000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>All!$B$257:$B$278</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="22"/>
+                <c:pt idx="0">
+                  <c:v>5.2258479562069899</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>5.1321123174082999</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>5.2437157298636796</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>5.2504871284328898</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5.2503356968257</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>5.2336543988027202</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>5.2591832551717097</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>5.2469052817766597</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>5.25892843081182</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>5.21286007784256</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>5.2596778259212398</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>5.2590212289624798</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>5.2296998738747797</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>5.2667771366869696</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>5.2271473404603404</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>5.2172814151544804</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>5.2026205255307998</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>5.2088502809019603</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>5.2306348705772896</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>5.2252366536496302</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>5.2416884024595696</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>5.2293252887733699</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>All!$C$257:$C$278</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="22"/>
+                <c:pt idx="0">
+                  <c:v>0.107867853594575</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.107552731189269</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.10779387708665</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.108339047437144</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.107577120583375</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.108317067772985</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.108753685676204</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.107673177325291</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.108229705876452</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.10760496944564001</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.108210284447238</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.108391645730674</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.10781058117576001</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.108326143627196</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.107921570762375</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0.107638855603815</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0.10699058330880699</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0.10798594921653699</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0.107583539743761</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>0.108049349994359</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>0.107467389213943</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>0.10771292800641501</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-0A5E-41D6-B680-57131B471AE9}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -12101,7 +12665,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4EAAD8A8-384F-4377-BC44-2ABC2E3B55D8}">
-  <dimension ref="A1:N228"/>
+  <dimension ref="A1:N278"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:14" ht="30" x14ac:dyDescent="0.25">
@@ -14687,6 +15251,556 @@
       </c>
       <c r="C228" s="1">
         <v>4.0347554180400501E-2</v>
+      </c>
+    </row>
+    <row r="229" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A229" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="B229" s="1">
+        <v>4.0279639492061596</v>
+      </c>
+      <c r="C229" s="1">
+        <v>8.3409466599106696E-2</v>
+      </c>
+    </row>
+    <row r="230" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A230" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="B230" s="1">
+        <v>4.0667523488381301</v>
+      </c>
+      <c r="C230" s="1">
+        <v>8.3177485471750606E-2</v>
+      </c>
+    </row>
+    <row r="231" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A231" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="B231" s="1">
+        <v>4.0183878243548996</v>
+      </c>
+      <c r="C231" s="1">
+        <v>8.3006037660706203E-2</v>
+      </c>
+    </row>
+    <row r="232" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A232" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="B232" s="1">
+        <v>4.0314213938624102</v>
+      </c>
+      <c r="C232" s="1">
+        <v>8.3019038948826299E-2</v>
+      </c>
+    </row>
+    <row r="233" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A233" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B233" s="1">
+        <v>4.0505545969773804</v>
+      </c>
+      <c r="C233" s="1">
+        <v>8.3723462750931996E-2</v>
+      </c>
+    </row>
+    <row r="234" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A234" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="B234" s="1">
+        <v>4.0517862191438496</v>
+      </c>
+      <c r="C234" s="1">
+        <v>8.3608574512507694E-2</v>
+      </c>
+    </row>
+    <row r="235" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A235" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="B235" s="1">
+        <v>4.0424645012040497</v>
+      </c>
+      <c r="C235" s="1">
+        <v>8.3118939745191397E-2</v>
+      </c>
+    </row>
+    <row r="236" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A236" s="1" t="s">
+        <v>247</v>
+      </c>
+      <c r="B236" s="1">
+        <v>4.0243487276243002</v>
+      </c>
+      <c r="C236" s="1">
+        <v>8.3605447355610901E-2</v>
+      </c>
+    </row>
+    <row r="237" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A237" s="1" t="s">
+        <v>248</v>
+      </c>
+      <c r="B237" s="1">
+        <v>4.0367409025359304</v>
+      </c>
+      <c r="C237" s="1">
+        <v>8.3418150740260003E-2</v>
+      </c>
+    </row>
+    <row r="238" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A238" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="B238" s="1">
+        <v>4.0491156124478902</v>
+      </c>
+      <c r="C238" s="1">
+        <v>8.3455841721042895E-2</v>
+      </c>
+    </row>
+    <row r="239" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A239" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="B239" s="1">
+        <v>4.0406778045491096</v>
+      </c>
+      <c r="C239" s="1">
+        <v>8.3276939213918696E-2</v>
+      </c>
+    </row>
+    <row r="240" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A240" s="1" t="s">
+        <v>251</v>
+      </c>
+      <c r="B240" s="1">
+        <v>4.0437611760653196</v>
+      </c>
+      <c r="C240" s="1">
+        <v>8.3116670967641595E-2</v>
+      </c>
+    </row>
+    <row r="241" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A241" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="B241" s="1">
+        <v>4.0356877834891698</v>
+      </c>
+      <c r="C241" s="1">
+        <v>8.3363484131550397E-2</v>
+      </c>
+    </row>
+    <row r="242" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A242" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="B242" s="1">
+        <v>4.0543291932026699</v>
+      </c>
+      <c r="C242" s="1">
+        <v>8.3757021233168596E-2</v>
+      </c>
+    </row>
+    <row r="243" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A243" s="1" t="s">
+        <v>254</v>
+      </c>
+      <c r="B243" s="1">
+        <v>4.0440448461837999</v>
+      </c>
+      <c r="C243" s="1">
+        <v>8.3417811249936594E-2</v>
+      </c>
+    </row>
+    <row r="244" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A244" s="1" t="s">
+        <v>255</v>
+      </c>
+      <c r="B244" s="1">
+        <v>4.0482658159189198</v>
+      </c>
+      <c r="C244" s="1">
+        <v>8.4025870340482506E-2</v>
+      </c>
+    </row>
+    <row r="245" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A245" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="B245" s="1">
+        <v>4.0372658698111801</v>
+      </c>
+      <c r="C245" s="1">
+        <v>8.2022959476588206E-2</v>
+      </c>
+    </row>
+    <row r="246" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A246" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="B246" s="1">
+        <v>4.0430873829414802</v>
+      </c>
+      <c r="C246" s="1">
+        <v>8.3225256404970693E-2</v>
+      </c>
+    </row>
+    <row r="247" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A247" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="B247" s="1">
+        <v>4.0311378792119203</v>
+      </c>
+      <c r="C247" s="1">
+        <v>8.2797901589345094E-2</v>
+      </c>
+    </row>
+    <row r="248" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A248" s="1" t="s">
+        <v>259</v>
+      </c>
+      <c r="B248" s="1">
+        <v>4.01331392262989</v>
+      </c>
+      <c r="C248" s="1">
+        <v>8.4124029452458504E-2</v>
+      </c>
+    </row>
+    <row r="249" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A249" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="B249" s="1">
+        <v>4.0578910745577002</v>
+      </c>
+      <c r="C249" s="1">
+        <v>8.2524964266572395E-2</v>
+      </c>
+    </row>
+    <row r="250" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A250" s="1" t="s">
+        <v>261</v>
+      </c>
+      <c r="B250" s="1">
+        <v>4.02794326730218</v>
+      </c>
+      <c r="C250" s="1">
+        <v>8.3779837646985295E-2</v>
+      </c>
+    </row>
+    <row r="251" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A251" s="1" t="s">
+        <v>262</v>
+      </c>
+      <c r="B251" s="1">
+        <v>4.0616651770599299</v>
+      </c>
+      <c r="C251" s="1">
+        <v>8.2884597799815607E-2</v>
+      </c>
+    </row>
+    <row r="252" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A252" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="B252" s="1">
+        <v>4.02065487780051</v>
+      </c>
+      <c r="C252" s="1">
+        <v>8.3056026546302203E-2</v>
+      </c>
+    </row>
+    <row r="253" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A253" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="B253" s="1">
+        <v>4.0194143809069702</v>
+      </c>
+      <c r="C253" s="1">
+        <v>8.3119909910801301E-2</v>
+      </c>
+    </row>
+    <row r="254" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A254" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="B254" s="1">
+        <v>4.0195181922825496</v>
+      </c>
+      <c r="C254" s="1">
+        <v>8.29152163470048E-2</v>
+      </c>
+    </row>
+    <row r="255" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A255" s="1" t="s">
+        <v>266</v>
+      </c>
+      <c r="B255" s="1">
+        <v>4.0060394450385299</v>
+      </c>
+      <c r="C255" s="1">
+        <v>8.28084692004942E-2</v>
+      </c>
+    </row>
+    <row r="256" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A256" s="1" t="s">
+        <v>267</v>
+      </c>
+      <c r="B256" s="1">
+        <v>4.03113906858741</v>
+      </c>
+      <c r="C256" s="1">
+        <v>8.3334028420614895E-2</v>
+      </c>
+    </row>
+    <row r="257" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A257" s="1" t="s">
+        <v>268</v>
+      </c>
+      <c r="B257" s="1">
+        <v>5.2258479562069899</v>
+      </c>
+      <c r="C257" s="1">
+        <v>0.107867853594575</v>
+      </c>
+    </row>
+    <row r="258" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A258" s="1" t="s">
+        <v>269</v>
+      </c>
+      <c r="B258" s="1">
+        <v>5.1321123174082999</v>
+      </c>
+      <c r="C258" s="1">
+        <v>0.107552731189269</v>
+      </c>
+    </row>
+    <row r="259" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A259" s="1" t="s">
+        <v>270</v>
+      </c>
+      <c r="B259" s="1">
+        <v>5.2437157298636796</v>
+      </c>
+      <c r="C259" s="1">
+        <v>0.10779387708665</v>
+      </c>
+    </row>
+    <row r="260" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A260" s="1" t="s">
+        <v>271</v>
+      </c>
+      <c r="B260" s="1">
+        <v>5.2504871284328898</v>
+      </c>
+      <c r="C260" s="1">
+        <v>0.108339047437144</v>
+      </c>
+    </row>
+    <row r="261" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A261" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="B261" s="1">
+        <v>5.2503356968257</v>
+      </c>
+      <c r="C261" s="1">
+        <v>0.107577120583375</v>
+      </c>
+    </row>
+    <row r="262" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A262" s="1" t="s">
+        <v>273</v>
+      </c>
+      <c r="B262" s="1">
+        <v>5.2336543988027202</v>
+      </c>
+      <c r="C262" s="1">
+        <v>0.108317067772985</v>
+      </c>
+    </row>
+    <row r="263" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A263" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="B263" s="1">
+        <v>5.2591832551717097</v>
+      </c>
+      <c r="C263" s="1">
+        <v>0.108753685676204</v>
+      </c>
+    </row>
+    <row r="264" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A264" s="1" t="s">
+        <v>275</v>
+      </c>
+      <c r="B264" s="1">
+        <v>5.2469052817766597</v>
+      </c>
+      <c r="C264" s="1">
+        <v>0.107673177325291</v>
+      </c>
+    </row>
+    <row r="265" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A265" s="1" t="s">
+        <v>276</v>
+      </c>
+      <c r="B265" s="1">
+        <v>5.25892843081182</v>
+      </c>
+      <c r="C265" s="1">
+        <v>0.108229705876452</v>
+      </c>
+    </row>
+    <row r="266" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A266" s="1" t="s">
+        <v>277</v>
+      </c>
+      <c r="B266" s="1">
+        <v>5.21286007784256</v>
+      </c>
+      <c r="C266" s="1">
+        <v>0.10760496944564001</v>
+      </c>
+    </row>
+    <row r="267" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A267" s="1" t="s">
+        <v>278</v>
+      </c>
+      <c r="B267" s="1">
+        <v>5.2596778259212398</v>
+      </c>
+      <c r="C267" s="1">
+        <v>0.108210284447238</v>
+      </c>
+    </row>
+    <row r="268" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A268" s="1" t="s">
+        <v>279</v>
+      </c>
+      <c r="B268" s="1">
+        <v>5.2590212289624798</v>
+      </c>
+      <c r="C268" s="1">
+        <v>0.108391645730674</v>
+      </c>
+    </row>
+    <row r="269" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A269" s="1" t="s">
+        <v>280</v>
+      </c>
+      <c r="B269" s="1">
+        <v>5.2296998738747797</v>
+      </c>
+      <c r="C269" s="1">
+        <v>0.10781058117576001</v>
+      </c>
+    </row>
+    <row r="270" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A270" s="1" t="s">
+        <v>281</v>
+      </c>
+      <c r="B270" s="1">
+        <v>5.2667771366869696</v>
+      </c>
+      <c r="C270" s="1">
+        <v>0.108326143627196</v>
+      </c>
+    </row>
+    <row r="271" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A271" s="1" t="s">
+        <v>282</v>
+      </c>
+      <c r="B271" s="1">
+        <v>5.2271473404603404</v>
+      </c>
+      <c r="C271" s="1">
+        <v>0.107921570762375</v>
+      </c>
+    </row>
+    <row r="272" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A272" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="B272" s="1">
+        <v>5.2172814151544804</v>
+      </c>
+      <c r="C272" s="1">
+        <v>0.107638855603815</v>
+      </c>
+    </row>
+    <row r="273" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A273" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="B273" s="1">
+        <v>5.2026205255307998</v>
+      </c>
+      <c r="C273" s="1">
+        <v>0.10699058330880699</v>
+      </c>
+    </row>
+    <row r="274" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A274" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="B274" s="1">
+        <v>5.2088502809019603</v>
+      </c>
+      <c r="C274" s="1">
+        <v>0.10798594921653699</v>
+      </c>
+    </row>
+    <row r="275" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A275" s="1" t="s">
+        <v>286</v>
+      </c>
+      <c r="B275" s="1">
+        <v>5.2306348705772896</v>
+      </c>
+      <c r="C275" s="1">
+        <v>0.107583539743761</v>
+      </c>
+    </row>
+    <row r="276" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A276" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="B276" s="1">
+        <v>5.2252366536496302</v>
+      </c>
+      <c r="C276" s="1">
+        <v>0.108049349994359</v>
+      </c>
+    </row>
+    <row r="277" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A277" s="1" t="s">
+        <v>288</v>
+      </c>
+      <c r="B277" s="1">
+        <v>5.2416884024595696</v>
+      </c>
+      <c r="C277" s="1">
+        <v>0.107467389213943</v>
+      </c>
+    </row>
+    <row r="278" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A278" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="B278" s="1">
+        <v>5.2293252887733699</v>
+      </c>
+      <c r="C278" s="1">
+        <v>0.10771292800641501</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Done with fitting data 1 more measurement day
</commit_message>
<xml_diff>
--- a/Fit Results/AllFitsF1=4.xlsx
+++ b/Fit Results/AllFitsF1=4.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Diego\git\6s7p\Fit Results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0DBB335-98CE-4F06-9EE6-88837AFDAE91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C416F13-A814-4B7A-983F-57B391AB54A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="All" sheetId="5" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="367" uniqueCount="349">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="421" uniqueCount="403">
   <si>
     <t>May22,2026+11-50-22AM</t>
   </si>
@@ -1086,6 +1086,168 @@
   </si>
   <si>
     <t>Jul16,2026+3-07-41PM</t>
+  </si>
+  <si>
+    <t>Jul17,2026+9-22-07AM</t>
+  </si>
+  <si>
+    <t>Jul17,2026+9-31-00AM</t>
+  </si>
+  <si>
+    <t>Jul17,2026+9-41-35AM</t>
+  </si>
+  <si>
+    <t>Jul17,2026+9-49-58AM</t>
+  </si>
+  <si>
+    <t>Jul17,2026+10-27-37AM</t>
+  </si>
+  <si>
+    <t>Jul17,2026+10-36-34AM</t>
+  </si>
+  <si>
+    <t>Jul17,2026+10-46-28AM</t>
+  </si>
+  <si>
+    <t>Jul17,2026+10-55-02AM</t>
+  </si>
+  <si>
+    <t>Jul17,2026+11-07-36AM</t>
+  </si>
+  <si>
+    <t>Jul17,2026+11-48-33AM</t>
+  </si>
+  <si>
+    <t>Jul17,2026+11-57-12AM</t>
+  </si>
+  <si>
+    <t>Jul17,2026+12-05-38PM</t>
+  </si>
+  <si>
+    <t>Jul17,2026+12-13-37PM</t>
+  </si>
+  <si>
+    <t>Jul17,2026+12-23-46PM</t>
+  </si>
+  <si>
+    <t>Jul17,2026+12-32-11PM</t>
+  </si>
+  <si>
+    <t>Jul17,2026+12-40-09PM</t>
+  </si>
+  <si>
+    <t>Jul17,2026+12-55-22PM</t>
+  </si>
+  <si>
+    <t>Jul17,2026+1-03-13PM</t>
+  </si>
+  <si>
+    <t>Jul17,2026+1-11-44PM</t>
+  </si>
+  <si>
+    <t>Jul17,2026+1-20-36PM</t>
+  </si>
+  <si>
+    <t>Jul17,2026+1-29-25PM</t>
+  </si>
+  <si>
+    <t>Jul17,2026+1-58-46PM</t>
+  </si>
+  <si>
+    <t>Jul17,2026+2-36-50PM</t>
+  </si>
+  <si>
+    <t>Jul17,2026+2-55-06PM</t>
+  </si>
+  <si>
+    <t>Jul20,2026+8-55-20AM</t>
+  </si>
+  <si>
+    <t>Jul20,2026+9-11-06AM</t>
+  </si>
+  <si>
+    <t>Jul20,2026+9-22-21AM</t>
+  </si>
+  <si>
+    <t>Jul20,2026+9-31-37AM</t>
+  </si>
+  <si>
+    <t>Jul20,2026+9-39-29AM</t>
+  </si>
+  <si>
+    <t>Jul20,2026+9-47-32AM</t>
+  </si>
+  <si>
+    <t>Jul20,2026+10-12-30AM</t>
+  </si>
+  <si>
+    <t>Jul20,2026+10-41-07AM</t>
+  </si>
+  <si>
+    <t>Jul20,2026+10-50-14AM</t>
+  </si>
+  <si>
+    <t>Jul20,2026+11-07-43AM</t>
+  </si>
+  <si>
+    <t>Jul20,2026+11-22-46AM</t>
+  </si>
+  <si>
+    <t>Jul20,2026+11-34-16AM</t>
+  </si>
+  <si>
+    <t>Jul20,2026+12-00-50PM</t>
+  </si>
+  <si>
+    <t>Jul20,2026+12-08-44PM</t>
+  </si>
+  <si>
+    <t>Jul20,2026+12-16-50PM</t>
+  </si>
+  <si>
+    <t>Jul20,2026+12-36-12PM</t>
+  </si>
+  <si>
+    <t>Jul20,2026+12-46-27PM</t>
+  </si>
+  <si>
+    <t>Jul20,2026+12-54-20PM</t>
+  </si>
+  <si>
+    <t>Jul20,2026+1-02-19PM</t>
+  </si>
+  <si>
+    <t>Jul20,2026+1-10-02PM</t>
+  </si>
+  <si>
+    <t>Jul20,2026+1-17-52PM</t>
+  </si>
+  <si>
+    <t>Jul20,2026+1-25-36PM</t>
+  </si>
+  <si>
+    <t>Jul20,2026+1-46-04PM</t>
+  </si>
+  <si>
+    <t>Jul20,2026+2-51-19PM</t>
+  </si>
+  <si>
+    <t>Jul20,2026+3-10-27PM</t>
+  </si>
+  <si>
+    <t>Jul20,2026+3-25-37PM</t>
+  </si>
+  <si>
+    <t>Jul20,2026+3-39-36PM</t>
+  </si>
+  <si>
+    <t>Jul20,2026+3-47-19PM</t>
+  </si>
+  <si>
+    <t>Jul20,2026+4-00-07PM</t>
+  </si>
+  <si>
+    <t>Jul20,2026+4-10-22PM</t>
   </si>
 </sst>
 </file>
@@ -3960,6 +4122,448 @@
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000001-E04E-4239-AE72-E247FFFE8129}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="14"/>
+          <c:order val="14"/>
+          <c:tx>
+            <c:v>17-Jul</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3">
+                  <a:lumMod val="80000"/>
+                  <a:lumOff val="20000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent3">
+                    <a:lumMod val="80000"/>
+                    <a:lumOff val="20000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>All!$B$338:$B$361</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="24"/>
+                <c:pt idx="0">
+                  <c:v>6.5540355078319896</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>6.5827244241657299</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>6.6067856280796899</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>6.5726574723992401</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>6.60849329589227</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>6.61449436632694</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>6.5773613187522404</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>6.6014893245484396</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>6.5572879597699503</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>6.6008191975600301</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>6.6252507343515497</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>6.5704906061544399</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>6.5936568893976704</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>6.5983973262679001</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>6.6115893763595901</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>6.5582265339750796</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>6.5712631537936099</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>6.6270719261065301</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>6.6192410240628501</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>6.57641937555222</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>6.6087667968385899</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>6.5350348620169401</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>6.5557760188699499</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>6.5032195210687904</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>All!$C$338:$C$361</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="24"/>
+                <c:pt idx="0">
+                  <c:v>0.105551348978041</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.105991123494967</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.10533604175596301</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.105665444142923</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.105198678205429</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.105495395727284</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.105314548416934</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.10568145895007799</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.10527614250211299</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.10576449952939899</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.10568293315542</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.10581148690660699</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.105635832709833</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.105645315996043</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.105275447604903</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0.105662668847811</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0.105625257618033</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0.106115800022815</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0.106389444933465</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>0.105686237933491</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>0.106107125977925</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>0.10569305527527301</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>0.105721916432143</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>0.10501733793063001</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-8960-4FD8-864C-A05C95AA4FC9}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="15"/>
+          <c:order val="15"/>
+          <c:tx>
+            <c:v>20-Jul</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent4">
+                  <a:lumMod val="80000"/>
+                  <a:lumOff val="20000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent4">
+                    <a:lumMod val="80000"/>
+                    <a:lumOff val="20000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>All!$B$362:$B$391</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="30"/>
+                <c:pt idx="0">
+                  <c:v>5.9622611291336396</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>6.0066466306228703</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>5.9421219928096498</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>5.97435305885893</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5.9503505932316996</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>5.9548297693894297</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>5.9553030366034303</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>5.9714415945772101</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>5.9546595386126704</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>5.9526717332290202</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>5.9925762983853099</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>5.9607737827043099</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>5.9798136479539004</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>5.9855117155737396</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>6.0292733180363696</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>5.9440797542562098</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>5.9637069175640898</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>5.9851248839214604</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>5.9753311000708296</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>5.95595351810669</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>5.9436339167314696</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>5.9680724903054401</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>5.97890051441588</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>5.9641145262355701</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>5.9548137587277301</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>5.9412161279185698</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>5.9237749973025897</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>5.9321677454244002</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>5.9655682681986404</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>5.9648566611082501</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>All!$C$362:$C$391</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="30"/>
+                <c:pt idx="0">
+                  <c:v>9.4951214409789694E-2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>9.48427612752826E-2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>9.5323780436117694E-2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>9.5239680372887395E-2</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>9.4913957126963905E-2</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>9.5207811574283305E-2</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>9.5333549341072299E-2</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>9.5272929905971096E-2</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>9.5825730092529093E-2</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>9.5557760398135405E-2</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>9.5707695616314301E-2</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>9.5513472864986904E-2</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>9.5307639125115001E-2</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>9.6102530139334702E-2</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>9.5842612321962603E-2</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>9.5502184039375396E-2</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>9.5885385701222001E-2</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>9.6439591076729503E-2</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>9.5315139971463694E-2</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>9.5613752572800206E-2</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>9.57329103303277E-2</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>9.4740461511437099E-2</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>9.56068005906138E-2</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>9.5241121615471297E-2</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>9.5433597155929403E-2</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>9.5987289369727502E-2</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>9.5313166809118E-2</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>9.5108590519696196E-2</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>9.5279653817559096E-2</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>9.5070431421425905E-2</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-8960-4FD8-864C-A05C95AA4FC9}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -12860,16 +13464,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>238124</xdr:colOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>609599</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>400050</xdr:rowOff>
+      <xdr:rowOff>133350</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>33</xdr:col>
-      <xdr:colOff>438150</xdr:colOff>
+      <xdr:col>31</xdr:col>
+      <xdr:colOff>200025</xdr:colOff>
       <xdr:row>16</xdr:row>
-      <xdr:rowOff>539750</xdr:rowOff>
+      <xdr:rowOff>273050</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -13314,7 +13918,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4EAAD8A8-384F-4377-BC44-2ABC2E3B55D8}">
-  <dimension ref="A1:N337"/>
+  <dimension ref="A1:N391"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:14" ht="30" x14ac:dyDescent="0.25">
@@ -17099,6 +17703,600 @@
       </c>
       <c r="C337" s="1">
         <v>6.3641331008131394E-2</v>
+      </c>
+    </row>
+    <row r="338" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A338" s="1" t="s">
+        <v>349</v>
+      </c>
+      <c r="B338" s="1">
+        <v>6.5540355078319896</v>
+      </c>
+      <c r="C338" s="1">
+        <v>0.105551348978041</v>
+      </c>
+    </row>
+    <row r="339" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A339" s="1" t="s">
+        <v>350</v>
+      </c>
+      <c r="B339" s="1">
+        <v>6.5827244241657299</v>
+      </c>
+      <c r="C339" s="1">
+        <v>0.105991123494967</v>
+      </c>
+    </row>
+    <row r="340" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A340" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="B340" s="1">
+        <v>6.6067856280796899</v>
+      </c>
+      <c r="C340" s="1">
+        <v>0.10533604175596301</v>
+      </c>
+    </row>
+    <row r="341" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A341" s="1" t="s">
+        <v>352</v>
+      </c>
+      <c r="B341" s="1">
+        <v>6.5726574723992401</v>
+      </c>
+      <c r="C341" s="1">
+        <v>0.105665444142923</v>
+      </c>
+    </row>
+    <row r="342" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A342" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="B342" s="1">
+        <v>6.60849329589227</v>
+      </c>
+      <c r="C342" s="1">
+        <v>0.105198678205429</v>
+      </c>
+    </row>
+    <row r="343" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A343" s="1" t="s">
+        <v>354</v>
+      </c>
+      <c r="B343" s="1">
+        <v>6.61449436632694</v>
+      </c>
+      <c r="C343" s="1">
+        <v>0.105495395727284</v>
+      </c>
+    </row>
+    <row r="344" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A344" s="1" t="s">
+        <v>355</v>
+      </c>
+      <c r="B344" s="1">
+        <v>6.5773613187522404</v>
+      </c>
+      <c r="C344" s="1">
+        <v>0.105314548416934</v>
+      </c>
+    </row>
+    <row r="345" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A345" s="1" t="s">
+        <v>356</v>
+      </c>
+      <c r="B345" s="1">
+        <v>6.6014893245484396</v>
+      </c>
+      <c r="C345" s="1">
+        <v>0.10568145895007799</v>
+      </c>
+    </row>
+    <row r="346" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A346" s="1" t="s">
+        <v>357</v>
+      </c>
+      <c r="B346" s="1">
+        <v>6.5572879597699503</v>
+      </c>
+      <c r="C346" s="1">
+        <v>0.10527614250211299</v>
+      </c>
+    </row>
+    <row r="347" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A347" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="B347" s="1">
+        <v>6.6008191975600301</v>
+      </c>
+      <c r="C347" s="1">
+        <v>0.10576449952939899</v>
+      </c>
+    </row>
+    <row r="348" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A348" s="1" t="s">
+        <v>359</v>
+      </c>
+      <c r="B348" s="1">
+        <v>6.6252507343515497</v>
+      </c>
+      <c r="C348" s="1">
+        <v>0.10568293315542</v>
+      </c>
+    </row>
+    <row r="349" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A349" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="B349" s="1">
+        <v>6.5704906061544399</v>
+      </c>
+      <c r="C349" s="1">
+        <v>0.10581148690660699</v>
+      </c>
+    </row>
+    <row r="350" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A350" s="1" t="s">
+        <v>361</v>
+      </c>
+      <c r="B350" s="1">
+        <v>6.5936568893976704</v>
+      </c>
+      <c r="C350" s="1">
+        <v>0.105635832709833</v>
+      </c>
+    </row>
+    <row r="351" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A351" s="1" t="s">
+        <v>362</v>
+      </c>
+      <c r="B351" s="1">
+        <v>6.5983973262679001</v>
+      </c>
+      <c r="C351" s="1">
+        <v>0.105645315996043</v>
+      </c>
+    </row>
+    <row r="352" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A352" s="1" t="s">
+        <v>363</v>
+      </c>
+      <c r="B352" s="1">
+        <v>6.6115893763595901</v>
+      </c>
+      <c r="C352" s="1">
+        <v>0.105275447604903</v>
+      </c>
+    </row>
+    <row r="353" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A353" s="1" t="s">
+        <v>364</v>
+      </c>
+      <c r="B353" s="1">
+        <v>6.5582265339750796</v>
+      </c>
+      <c r="C353" s="1">
+        <v>0.105662668847811</v>
+      </c>
+    </row>
+    <row r="354" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A354" s="1" t="s">
+        <v>365</v>
+      </c>
+      <c r="B354" s="1">
+        <v>6.5712631537936099</v>
+      </c>
+      <c r="C354" s="1">
+        <v>0.105625257618033</v>
+      </c>
+    </row>
+    <row r="355" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A355" s="1" t="s">
+        <v>366</v>
+      </c>
+      <c r="B355" s="1">
+        <v>6.6270719261065301</v>
+      </c>
+      <c r="C355" s="1">
+        <v>0.106115800022815</v>
+      </c>
+    </row>
+    <row r="356" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A356" s="1" t="s">
+        <v>367</v>
+      </c>
+      <c r="B356" s="1">
+        <v>6.6192410240628501</v>
+      </c>
+      <c r="C356" s="1">
+        <v>0.106389444933465</v>
+      </c>
+    </row>
+    <row r="357" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A357" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="B357" s="1">
+        <v>6.57641937555222</v>
+      </c>
+      <c r="C357" s="1">
+        <v>0.105686237933491</v>
+      </c>
+    </row>
+    <row r="358" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A358" s="1" t="s">
+        <v>369</v>
+      </c>
+      <c r="B358" s="1">
+        <v>6.6087667968385899</v>
+      </c>
+      <c r="C358" s="1">
+        <v>0.106107125977925</v>
+      </c>
+    </row>
+    <row r="359" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A359" s="1" t="s">
+        <v>370</v>
+      </c>
+      <c r="B359" s="1">
+        <v>6.5350348620169401</v>
+      </c>
+      <c r="C359" s="1">
+        <v>0.10569305527527301</v>
+      </c>
+    </row>
+    <row r="360" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A360" s="1" t="s">
+        <v>371</v>
+      </c>
+      <c r="B360" s="1">
+        <v>6.5557760188699499</v>
+      </c>
+      <c r="C360" s="1">
+        <v>0.105721916432143</v>
+      </c>
+    </row>
+    <row r="361" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A361" s="1" t="s">
+        <v>372</v>
+      </c>
+      <c r="B361" s="1">
+        <v>6.5032195210687904</v>
+      </c>
+      <c r="C361" s="1">
+        <v>0.10501733793063001</v>
+      </c>
+    </row>
+    <row r="362" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A362" s="1" t="s">
+        <v>373</v>
+      </c>
+      <c r="B362" s="1">
+        <v>5.9622611291336396</v>
+      </c>
+      <c r="C362" s="1">
+        <v>9.4951214409789694E-2</v>
+      </c>
+    </row>
+    <row r="363" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A363" s="1" t="s">
+        <v>374</v>
+      </c>
+      <c r="B363" s="1">
+        <v>6.0066466306228703</v>
+      </c>
+      <c r="C363" s="1">
+        <v>9.48427612752826E-2</v>
+      </c>
+    </row>
+    <row r="364" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A364" s="1" t="s">
+        <v>375</v>
+      </c>
+      <c r="B364" s="1">
+        <v>5.9421219928096498</v>
+      </c>
+      <c r="C364" s="1">
+        <v>9.5323780436117694E-2</v>
+      </c>
+    </row>
+    <row r="365" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A365" s="1" t="s">
+        <v>376</v>
+      </c>
+      <c r="B365" s="1">
+        <v>5.97435305885893</v>
+      </c>
+      <c r="C365" s="1">
+        <v>9.5239680372887395E-2</v>
+      </c>
+    </row>
+    <row r="366" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A366" s="1" t="s">
+        <v>377</v>
+      </c>
+      <c r="B366" s="1">
+        <v>5.9503505932316996</v>
+      </c>
+      <c r="C366" s="1">
+        <v>9.4913957126963905E-2</v>
+      </c>
+    </row>
+    <row r="367" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A367" s="1" t="s">
+        <v>378</v>
+      </c>
+      <c r="B367" s="1">
+        <v>5.9548297693894297</v>
+      </c>
+      <c r="C367" s="1">
+        <v>9.5207811574283305E-2</v>
+      </c>
+    </row>
+    <row r="368" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A368" s="1" t="s">
+        <v>379</v>
+      </c>
+      <c r="B368" s="1">
+        <v>5.9553030366034303</v>
+      </c>
+      <c r="C368" s="1">
+        <v>9.5333549341072299E-2</v>
+      </c>
+    </row>
+    <row r="369" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A369" s="1" t="s">
+        <v>380</v>
+      </c>
+      <c r="B369" s="1">
+        <v>5.9714415945772101</v>
+      </c>
+      <c r="C369" s="1">
+        <v>9.5272929905971096E-2</v>
+      </c>
+    </row>
+    <row r="370" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A370" s="1" t="s">
+        <v>381</v>
+      </c>
+      <c r="B370" s="1">
+        <v>5.9546595386126704</v>
+      </c>
+      <c r="C370" s="1">
+        <v>9.5825730092529093E-2</v>
+      </c>
+    </row>
+    <row r="371" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A371" s="1" t="s">
+        <v>382</v>
+      </c>
+      <c r="B371" s="1">
+        <v>5.9526717332290202</v>
+      </c>
+      <c r="C371" s="1">
+        <v>9.5557760398135405E-2</v>
+      </c>
+    </row>
+    <row r="372" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A372" s="1" t="s">
+        <v>383</v>
+      </c>
+      <c r="B372" s="1">
+        <v>5.9925762983853099</v>
+      </c>
+      <c r="C372" s="1">
+        <v>9.5707695616314301E-2</v>
+      </c>
+    </row>
+    <row r="373" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A373" s="1" t="s">
+        <v>384</v>
+      </c>
+      <c r="B373" s="1">
+        <v>5.9607737827043099</v>
+      </c>
+      <c r="C373" s="1">
+        <v>9.5513472864986904E-2</v>
+      </c>
+    </row>
+    <row r="374" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A374" s="1" t="s">
+        <v>385</v>
+      </c>
+      <c r="B374" s="1">
+        <v>5.9798136479539004</v>
+      </c>
+      <c r="C374" s="1">
+        <v>9.5307639125115001E-2</v>
+      </c>
+    </row>
+    <row r="375" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A375" s="1" t="s">
+        <v>386</v>
+      </c>
+      <c r="B375" s="1">
+        <v>5.9855117155737396</v>
+      </c>
+      <c r="C375" s="1">
+        <v>9.6102530139334702E-2</v>
+      </c>
+    </row>
+    <row r="376" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A376" s="1" t="s">
+        <v>387</v>
+      </c>
+      <c r="B376" s="1">
+        <v>6.0292733180363696</v>
+      </c>
+      <c r="C376" s="1">
+        <v>9.5842612321962603E-2</v>
+      </c>
+    </row>
+    <row r="377" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A377" s="1" t="s">
+        <v>388</v>
+      </c>
+      <c r="B377" s="1">
+        <v>5.9440797542562098</v>
+      </c>
+      <c r="C377" s="1">
+        <v>9.5502184039375396E-2</v>
+      </c>
+    </row>
+    <row r="378" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A378" s="1" t="s">
+        <v>389</v>
+      </c>
+      <c r="B378" s="1">
+        <v>5.9637069175640898</v>
+      </c>
+      <c r="C378" s="1">
+        <v>9.5885385701222001E-2</v>
+      </c>
+    </row>
+    <row r="379" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A379" s="1" t="s">
+        <v>390</v>
+      </c>
+      <c r="B379" s="1">
+        <v>5.9851248839214604</v>
+      </c>
+      <c r="C379" s="1">
+        <v>9.6439591076729503E-2</v>
+      </c>
+    </row>
+    <row r="380" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A380" s="1" t="s">
+        <v>391</v>
+      </c>
+      <c r="B380" s="1">
+        <v>5.9753311000708296</v>
+      </c>
+      <c r="C380" s="1">
+        <v>9.5315139971463694E-2</v>
+      </c>
+    </row>
+    <row r="381" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A381" s="1" t="s">
+        <v>392</v>
+      </c>
+      <c r="B381" s="1">
+        <v>5.95595351810669</v>
+      </c>
+      <c r="C381" s="1">
+        <v>9.5613752572800206E-2</v>
+      </c>
+    </row>
+    <row r="382" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A382" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="B382" s="1">
+        <v>5.9436339167314696</v>
+      </c>
+      <c r="C382" s="1">
+        <v>9.57329103303277E-2</v>
+      </c>
+    </row>
+    <row r="383" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A383" s="1" t="s">
+        <v>394</v>
+      </c>
+      <c r="B383" s="1">
+        <v>5.9680724903054401</v>
+      </c>
+      <c r="C383" s="1">
+        <v>9.4740461511437099E-2</v>
+      </c>
+    </row>
+    <row r="384" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A384" s="1" t="s">
+        <v>395</v>
+      </c>
+      <c r="B384" s="1">
+        <v>5.97890051441588</v>
+      </c>
+      <c r="C384" s="1">
+        <v>9.56068005906138E-2</v>
+      </c>
+    </row>
+    <row r="385" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A385" s="1" t="s">
+        <v>396</v>
+      </c>
+      <c r="B385" s="1">
+        <v>5.9641145262355701</v>
+      </c>
+      <c r="C385" s="1">
+        <v>9.5241121615471297E-2</v>
+      </c>
+    </row>
+    <row r="386" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A386" s="1" t="s">
+        <v>397</v>
+      </c>
+      <c r="B386" s="1">
+        <v>5.9548137587277301</v>
+      </c>
+      <c r="C386" s="1">
+        <v>9.5433597155929403E-2</v>
+      </c>
+    </row>
+    <row r="387" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A387" s="1" t="s">
+        <v>398</v>
+      </c>
+      <c r="B387" s="1">
+        <v>5.9412161279185698</v>
+      </c>
+      <c r="C387" s="1">
+        <v>9.5987289369727502E-2</v>
+      </c>
+    </row>
+    <row r="388" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A388" s="1" t="s">
+        <v>399</v>
+      </c>
+      <c r="B388" s="1">
+        <v>5.9237749973025897</v>
+      </c>
+      <c r="C388" s="1">
+        <v>9.5313166809118E-2</v>
+      </c>
+    </row>
+    <row r="389" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A389" s="1" t="s">
+        <v>400</v>
+      </c>
+      <c r="B389" s="1">
+        <v>5.9321677454244002</v>
+      </c>
+      <c r="C389" s="1">
+        <v>9.5108590519696196E-2</v>
+      </c>
+    </row>
+    <row r="390" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A390" s="1" t="s">
+        <v>401</v>
+      </c>
+      <c r="B390" s="1">
+        <v>5.9655682681986404</v>
+      </c>
+      <c r="C390" s="1">
+        <v>9.5279653817559096E-2</v>
+      </c>
+    </row>
+    <row r="391" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A391" s="1" t="s">
+        <v>402</v>
+      </c>
+      <c r="B391" s="1">
+        <v>5.9648566611082501</v>
+      </c>
+      <c r="C391" s="1">
+        <v>9.5070431421425905E-2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Need to rerun for quadratic 894 background
</commit_message>
<xml_diff>
--- a/Fit Results/AllFitsF1=4.xlsx
+++ b/Fit Results/AllFitsF1=4.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Diego\git\6s7p\Fit Results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C416F13-A814-4B7A-983F-57B391AB54A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A09B28F3-B141-4BFA-846C-FBC4A3F9103D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="All" sheetId="5" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="421" uniqueCount="403">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="451" uniqueCount="433">
   <si>
     <t>May22,2026+11-50-22AM</t>
   </si>
@@ -848,9 +848,6 @@
     <t>Jul14,2026+12-14-44PM</t>
   </si>
   <si>
-    <t>Jul14,2026+12-26-20PM</t>
-  </si>
-  <si>
     <t>Jul14,2026+12-34-37PM</t>
   </si>
   <si>
@@ -1157,9 +1154,6 @@
     <t>Jul17,2026+2-36-50PM</t>
   </si>
   <si>
-    <t>Jul17,2026+2-55-06PM</t>
-  </si>
-  <si>
     <t>Jul20,2026+8-55-20AM</t>
   </si>
   <si>
@@ -1248,6 +1242,102 @@
   </si>
   <si>
     <t>Jul20,2026+4-10-22PM</t>
+  </si>
+  <si>
+    <t>Jul21,2026+9-09-03AM</t>
+  </si>
+  <si>
+    <t>Jul21,2026+9-17-16AM</t>
+  </si>
+  <si>
+    <t>Jul21,2026+9-25-02AM</t>
+  </si>
+  <si>
+    <t>Jul21,2026+9-32-41AM</t>
+  </si>
+  <si>
+    <t>Jul21,2026+9-40-56AM</t>
+  </si>
+  <si>
+    <t>Jul21,2026+9-52-24AM</t>
+  </si>
+  <si>
+    <t>Jul21,2026+10-04-37AM</t>
+  </si>
+  <si>
+    <t>Jul21,2026+10-41-13AM</t>
+  </si>
+  <si>
+    <t>Jul21,2026+12-09-01PM</t>
+  </si>
+  <si>
+    <t>Jul21,2026+12-43-22PM</t>
+  </si>
+  <si>
+    <t>Jul21,2026+12-53-22PM</t>
+  </si>
+  <si>
+    <t>Jul21,2026+1-01-31PM</t>
+  </si>
+  <si>
+    <t>Jul21,2026+1-09-11PM</t>
+  </si>
+  <si>
+    <t>Jul21,2026+1-30-31PM</t>
+  </si>
+  <si>
+    <t>Jul21,2026+1-40-05PM</t>
+  </si>
+  <si>
+    <t>Jul21,2026+1-58-35PM</t>
+  </si>
+  <si>
+    <t>Jul21,2026+2-08-08PM</t>
+  </si>
+  <si>
+    <t>Jul21,2026+2-15-55PM</t>
+  </si>
+  <si>
+    <t>Jul21,2026+2-23-55PM</t>
+  </si>
+  <si>
+    <t>Jul21,2026+2-32-03PM</t>
+  </si>
+  <si>
+    <t>Jul21,2026+3-10-36PM</t>
+  </si>
+  <si>
+    <t>Jul21,2026+3-18-15PM</t>
+  </si>
+  <si>
+    <t>Jul21,2026+3-26-50PM</t>
+  </si>
+  <si>
+    <t>Jul21,2026+3-34-26PM</t>
+  </si>
+  <si>
+    <t>Jul21,2026+3-42-02PM</t>
+  </si>
+  <si>
+    <t>Jul21,2026+3-49-49PM</t>
+  </si>
+  <si>
+    <t>Jul21,2026+3-57-30PM</t>
+  </si>
+  <si>
+    <t>Jul21,2026+4-05-10PM</t>
+  </si>
+  <si>
+    <t>Jul21,2026+4-20-56PM</t>
+  </si>
+  <si>
+    <t>Jul21,2026+4-31-22PM</t>
+  </si>
+  <si>
+    <t>Jul21,2026+4-38-59PM</t>
+  </si>
+  <si>
+    <t>Jul21,2026+4-46-38PM</t>
   </si>
 </sst>
 </file>
@@ -3498,74 +3588,71 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>All!$B$257:$B$278</c:f>
+              <c:f>All!$B$257:$B$277</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="22"/>
+                <c:ptCount val="21"/>
                 <c:pt idx="0">
                   <c:v>5.2258479562069899</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>5.1321123174082999</c:v>
+                  <c:v>5.2437157298636796</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>5.2437157298636796</c:v>
+                  <c:v>5.2504871284328898</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5.2504871284328898</c:v>
+                  <c:v>5.2503356968257</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>5.2503356968257</c:v>
+                  <c:v>5.2336543988027202</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>5.2336543988027202</c:v>
+                  <c:v>5.2591832551717097</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>5.2591832551717097</c:v>
+                  <c:v>5.2469052817766597</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>5.2469052817766597</c:v>
+                  <c:v>5.25892843081182</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>5.25892843081182</c:v>
+                  <c:v>5.21286007784256</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>5.21286007784256</c:v>
+                  <c:v>5.2596778259212398</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>5.2596778259212398</c:v>
+                  <c:v>5.2590212289624798</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>5.2590212289624798</c:v>
+                  <c:v>5.2296998738747797</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>5.2296998738747797</c:v>
+                  <c:v>5.2667771366869696</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>5.2667771366869696</c:v>
+                  <c:v>5.2271473404603404</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>5.2271473404603404</c:v>
+                  <c:v>5.2172814151544804</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>5.2172814151544804</c:v>
+                  <c:v>5.2026205255307998</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>5.2026205255307998</c:v>
+                  <c:v>5.2088502809019603</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>5.2088502809019603</c:v>
+                  <c:v>5.2306348705772896</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>5.2306348705772896</c:v>
+                  <c:v>5.2252366536496302</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>5.2252366536496302</c:v>
+                  <c:v>5.2416884024595696</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>5.2416884024595696</c:v>
-                </c:pt>
-                <c:pt idx="21">
                   <c:v>5.2293252887733699</c:v>
                 </c:pt>
               </c:numCache>
@@ -3573,74 +3660,71 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>All!$C$257:$C$278</c:f>
+              <c:f>All!$C$257:$C$277</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="22"/>
+                <c:ptCount val="21"/>
                 <c:pt idx="0">
                   <c:v>8.4098670481367904E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>8.3770582022428597E-2</c:v>
+                  <c:v>8.3930571430078399E-2</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>8.3930571430078399E-2</c:v>
+                  <c:v>8.4386871474939104E-2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>8.4386871474939104E-2</c:v>
+                  <c:v>8.3779094698236606E-2</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>8.3779094698236606E-2</c:v>
+                  <c:v>8.4368245251587398E-2</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>8.4368245251587398E-2</c:v>
+                  <c:v>8.4640740114124396E-2</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>8.4640740114124396E-2</c:v>
+                  <c:v>8.3819572528152295E-2</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>8.3819572528152295E-2</c:v>
+                  <c:v>8.4298501986348195E-2</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>8.4298501986348195E-2</c:v>
+                  <c:v>8.3749879844150901E-2</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>8.3749879844150901E-2</c:v>
+                  <c:v>8.4288203419773597E-2</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>8.4288203419773597E-2</c:v>
+                  <c:v>8.4433783424020706E-2</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>8.4433783424020706E-2</c:v>
+                  <c:v>8.3978129655986694E-2</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>8.3978129655986694E-2</c:v>
+                  <c:v>8.4391376865179599E-2</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>8.4391376865179599E-2</c:v>
+                  <c:v>8.3986778727553404E-2</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>8.3986778727553404E-2</c:v>
+                  <c:v>8.3700704517771493E-2</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>8.3700704517771493E-2</c:v>
+                  <c:v>8.3337504828946599E-2</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>8.3337504828946599E-2</c:v>
+                  <c:v>8.4048471187493506E-2</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>8.4048471187493506E-2</c:v>
+                  <c:v>8.3859299335631896E-2</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>8.3859299335631896E-2</c:v>
+                  <c:v>8.4150599797561301E-2</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>8.4150599797561301E-2</c:v>
+                  <c:v>8.3705403747337398E-2</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>8.3705403747337398E-2</c:v>
-                </c:pt>
-                <c:pt idx="21">
                   <c:v>8.38953398940607E-2</c:v>
                 </c:pt>
               </c:numCache>
@@ -3689,7 +3773,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>All!$B$279:$B$302</c:f>
+              <c:f>All!$B$278:$B$301</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="24"/>
@@ -3770,7 +3854,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>All!$C$279:$C$302</c:f>
+              <c:f>All!$C$278:$C$301</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="24"/>
@@ -3892,7 +3976,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>All!$B$303:$B$337</c:f>
+              <c:f>All!$B$302:$B$336</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="35"/>
@@ -4006,7 +4090,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>All!$C$303:$C$337</c:f>
+              <c:f>All!$C$302:$C$336</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="35"/>
@@ -4161,10 +4245,10 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>All!$B$338:$B$361</c:f>
+              <c:f>All!$B$337:$B$359</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="24"/>
+                <c:ptCount val="23"/>
                 <c:pt idx="0">
                   <c:v>6.5540355078319896</c:v>
                 </c:pt>
@@ -4233,19 +4317,16 @@
                 </c:pt>
                 <c:pt idx="22">
                   <c:v>6.5557760188699499</c:v>
-                </c:pt>
-                <c:pt idx="23">
-                  <c:v>6.5032195210687904</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>All!$C$338:$C$361</c:f>
+              <c:f>All!$C$337:$C$359</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="24"/>
+                <c:ptCount val="23"/>
                 <c:pt idx="0">
                   <c:v>0.105551348978041</c:v>
                 </c:pt>
@@ -4314,9 +4395,6 @@
                 </c:pt>
                 <c:pt idx="22">
                   <c:v>0.105721916432143</c:v>
-                </c:pt>
-                <c:pt idx="23">
-                  <c:v>0.10501733793063001</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4364,7 +4442,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>All!$B$362:$B$391</c:f>
+              <c:f>All!$B$360:$B$389</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="30"/>
@@ -4463,7 +4541,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>All!$C$362:$C$391</c:f>
+              <c:f>All!$C$360:$C$389</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="30"/>
@@ -4564,6 +4642,257 @@
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000002-8960-4FD8-864C-A05C95AA4FC9}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="16"/>
+          <c:order val="16"/>
+          <c:tx>
+            <c:v>21-Jul</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent5">
+                  <a:lumMod val="80000"/>
+                  <a:lumOff val="20000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent5">
+                    <a:lumMod val="80000"/>
+                    <a:lumOff val="20000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>All!$B$390:$B$421</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="32"/>
+                <c:pt idx="0">
+                  <c:v>3.0672817324059798</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>3.06498328697809</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3.06753441554193</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3.0756019900176499</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>3.0649036050172098</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>3.06529341587372</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>3.0726606549971298</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>3.0831176610414701</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>3.0668965665752701</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>3.0577539539137901</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>3.0461287705788598</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>3.0420177016521102</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>3.0577648925430601</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>3.07207699092403</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>3.0603120961688499</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>3.0495273783215602</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>3.0483213432966099</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>3.0507028081060601</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>3.0503873160495498</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>3.0616213771126799</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>3.0441812745358798</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>3.0545733491419398</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>3.0565111313221198</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>3.0569612836170998</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>3.0531280697850698</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>3.0495276887412501</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>3.0451824247254602</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>3.0636069285517098</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>3.0573709331599099</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>3.0482345249944598</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>3.0486121479316401</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>3.0547580292283598</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>All!$C$390:$C$421</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="32"/>
+                <c:pt idx="0">
+                  <c:v>4.9220544832568401E-2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>4.8826525513616603E-2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>4.9256122272570202E-2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4.97179954883646E-2</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>4.9725118840505199E-2</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>4.9381962862556E-2</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>4.8979944321647401E-2</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>4.9045485231240298E-2</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>4.8965298287210399E-2</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>4.8957627310304702E-2</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>4.9000057015244597E-2</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>4.8651617087087401E-2</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>4.8810930819998197E-2</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>4.8901071369119802E-2</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>4.9126205451321202E-2</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>4.95058693259324E-2</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>4.8651769164606402E-2</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>4.8908241247632697E-2</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>4.8699146330509702E-2</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>4.91555175312548E-2</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>4.9268660787059597E-2</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>4.8826826414769098E-2</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>4.8764627198113697E-2</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>4.9029160899217702E-2</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>4.8854122518207498E-2</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>4.9133881801381701E-2</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>4.9071806924917999E-2</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>4.9142870700877098E-2</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>4.9249210174874901E-2</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>4.8951873888496603E-2</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>4.8933368456572202E-2</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>4.87619094275357E-2</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-E732-4D6D-A1BB-56358B21E154}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -13918,7 +14247,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4EAAD8A8-384F-4377-BC44-2ABC2E3B55D8}">
-  <dimension ref="A1:N391"/>
+  <dimension ref="A1:N421"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:14" ht="30" x14ac:dyDescent="0.25">
@@ -16830,10 +17159,10 @@
         <v>269</v>
       </c>
       <c r="B258" s="1">
-        <v>5.1321123174082999</v>
+        <v>5.2437157298636796</v>
       </c>
       <c r="C258" s="1">
-        <v>8.3770582022428597E-2</v>
+        <v>8.3930571430078399E-2</v>
       </c>
     </row>
     <row r="259" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -16841,10 +17170,10 @@
         <v>270</v>
       </c>
       <c r="B259" s="1">
-        <v>5.2437157298636796</v>
+        <v>5.2504871284328898</v>
       </c>
       <c r="C259" s="1">
-        <v>8.3930571430078399E-2</v>
+        <v>8.4386871474939104E-2</v>
       </c>
     </row>
     <row r="260" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -16852,10 +17181,10 @@
         <v>271</v>
       </c>
       <c r="B260" s="1">
-        <v>5.2504871284328898</v>
+        <v>5.2503356968257</v>
       </c>
       <c r="C260" s="1">
-        <v>8.4386871474939104E-2</v>
+        <v>8.3779094698236606E-2</v>
       </c>
     </row>
     <row r="261" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -16863,10 +17192,10 @@
         <v>272</v>
       </c>
       <c r="B261" s="1">
-        <v>5.2503356968257</v>
+        <v>5.2336543988027202</v>
       </c>
       <c r="C261" s="1">
-        <v>8.3779094698236606E-2</v>
+        <v>8.4368245251587398E-2</v>
       </c>
     </row>
     <row r="262" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -16874,10 +17203,10 @@
         <v>273</v>
       </c>
       <c r="B262" s="1">
-        <v>5.2336543988027202</v>
+        <v>5.2591832551717097</v>
       </c>
       <c r="C262" s="1">
-        <v>8.4368245251587398E-2</v>
+        <v>8.4640740114124396E-2</v>
       </c>
     </row>
     <row r="263" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -16885,10 +17214,10 @@
         <v>274</v>
       </c>
       <c r="B263" s="1">
-        <v>5.2591832551717097</v>
+        <v>5.2469052817766597</v>
       </c>
       <c r="C263" s="1">
-        <v>8.4640740114124396E-2</v>
+        <v>8.3819572528152295E-2</v>
       </c>
     </row>
     <row r="264" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -16896,10 +17225,10 @@
         <v>275</v>
       </c>
       <c r="B264" s="1">
-        <v>5.2469052817766597</v>
+        <v>5.25892843081182</v>
       </c>
       <c r="C264" s="1">
-        <v>8.3819572528152295E-2</v>
+        <v>8.4298501986348195E-2</v>
       </c>
     </row>
     <row r="265" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -16907,10 +17236,10 @@
         <v>276</v>
       </c>
       <c r="B265" s="1">
-        <v>5.25892843081182</v>
+        <v>5.21286007784256</v>
       </c>
       <c r="C265" s="1">
-        <v>8.4298501986348195E-2</v>
+        <v>8.3749879844150901E-2</v>
       </c>
     </row>
     <row r="266" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -16918,10 +17247,10 @@
         <v>277</v>
       </c>
       <c r="B266" s="1">
-        <v>5.21286007784256</v>
+        <v>5.2596778259212398</v>
       </c>
       <c r="C266" s="1">
-        <v>8.3749879844150901E-2</v>
+        <v>8.4288203419773597E-2</v>
       </c>
     </row>
     <row r="267" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -16929,10 +17258,10 @@
         <v>278</v>
       </c>
       <c r="B267" s="1">
-        <v>5.2596778259212398</v>
+        <v>5.2590212289624798</v>
       </c>
       <c r="C267" s="1">
-        <v>8.4288203419773597E-2</v>
+        <v>8.4433783424020706E-2</v>
       </c>
     </row>
     <row r="268" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -16940,10 +17269,10 @@
         <v>279</v>
       </c>
       <c r="B268" s="1">
-        <v>5.2590212289624798</v>
+        <v>5.2296998738747797</v>
       </c>
       <c r="C268" s="1">
-        <v>8.4433783424020706E-2</v>
+        <v>8.3978129655986694E-2</v>
       </c>
     </row>
     <row r="269" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -16951,10 +17280,10 @@
         <v>280</v>
       </c>
       <c r="B269" s="1">
-        <v>5.2296998738747797</v>
+        <v>5.2667771366869696</v>
       </c>
       <c r="C269" s="1">
-        <v>8.3978129655986694E-2</v>
+        <v>8.4391376865179599E-2</v>
       </c>
     </row>
     <row r="270" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -16962,10 +17291,10 @@
         <v>281</v>
       </c>
       <c r="B270" s="1">
-        <v>5.2667771366869696</v>
+        <v>5.2271473404603404</v>
       </c>
       <c r="C270" s="1">
-        <v>8.4391376865179599E-2</v>
+        <v>8.3986778727553404E-2</v>
       </c>
     </row>
     <row r="271" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -16973,10 +17302,10 @@
         <v>282</v>
       </c>
       <c r="B271" s="1">
-        <v>5.2271473404603404</v>
+        <v>5.2172814151544804</v>
       </c>
       <c r="C271" s="1">
-        <v>8.3986778727553404E-2</v>
+        <v>8.3700704517771493E-2</v>
       </c>
     </row>
     <row r="272" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -16984,10 +17313,10 @@
         <v>283</v>
       </c>
       <c r="B272" s="1">
-        <v>5.2172814151544804</v>
+        <v>5.2026205255307998</v>
       </c>
       <c r="C272" s="1">
-        <v>8.3700704517771493E-2</v>
+        <v>8.3337504828946599E-2</v>
       </c>
     </row>
     <row r="273" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -16995,10 +17324,10 @@
         <v>284</v>
       </c>
       <c r="B273" s="1">
-        <v>5.2026205255307998</v>
+        <v>5.2088502809019603</v>
       </c>
       <c r="C273" s="1">
-        <v>8.3337504828946599E-2</v>
+        <v>8.4048471187493506E-2</v>
       </c>
     </row>
     <row r="274" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17006,10 +17335,10 @@
         <v>285</v>
       </c>
       <c r="B274" s="1">
-        <v>5.2088502809019603</v>
+        <v>5.2306348705772896</v>
       </c>
       <c r="C274" s="1">
-        <v>8.4048471187493506E-2</v>
+        <v>8.3859299335631896E-2</v>
       </c>
     </row>
     <row r="275" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17017,10 +17346,10 @@
         <v>286</v>
       </c>
       <c r="B275" s="1">
-        <v>5.2306348705772896</v>
+        <v>5.2252366536496302</v>
       </c>
       <c r="C275" s="1">
-        <v>8.3859299335631896E-2</v>
+        <v>8.4150599797561301E-2</v>
       </c>
     </row>
     <row r="276" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17028,10 +17357,10 @@
         <v>287</v>
       </c>
       <c r="B276" s="1">
-        <v>5.2252366536496302</v>
+        <v>5.2416884024595696</v>
       </c>
       <c r="C276" s="1">
-        <v>8.4150599797561301E-2</v>
+        <v>8.3705403747337398E-2</v>
       </c>
     </row>
     <row r="277" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17039,10 +17368,10 @@
         <v>288</v>
       </c>
       <c r="B277" s="1">
-        <v>5.2416884024595696</v>
+        <v>5.2293252887733699</v>
       </c>
       <c r="C277" s="1">
-        <v>8.3705403747337398E-2</v>
+        <v>8.38953398940607E-2</v>
       </c>
     </row>
     <row r="278" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17050,10 +17379,10 @@
         <v>289</v>
       </c>
       <c r="B278" s="1">
-        <v>5.2293252887733699</v>
+        <v>5.2401573655099698</v>
       </c>
       <c r="C278" s="1">
-        <v>8.38953398940607E-2</v>
+        <v>8.4020421663362793E-2</v>
       </c>
     </row>
     <row r="279" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17061,10 +17390,10 @@
         <v>290</v>
       </c>
       <c r="B279" s="1">
-        <v>5.2401573655099698</v>
+        <v>5.2402095305102501</v>
       </c>
       <c r="C279" s="1">
-        <v>8.4020421663362793E-2</v>
+        <v>8.3856539409502107E-2</v>
       </c>
     </row>
     <row r="280" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17072,10 +17401,10 @@
         <v>291</v>
       </c>
       <c r="B280" s="1">
-        <v>5.2402095305102501</v>
+        <v>5.2325481598897898</v>
       </c>
       <c r="C280" s="1">
-        <v>8.3856539409502107E-2</v>
+        <v>8.4441497497705006E-2</v>
       </c>
     </row>
     <row r="281" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17083,10 +17412,10 @@
         <v>292</v>
       </c>
       <c r="B281" s="1">
-        <v>5.2325481598897898</v>
+        <v>5.2632048700287699</v>
       </c>
       <c r="C281" s="1">
-        <v>8.4441497497705006E-2</v>
+        <v>8.3922207540377103E-2</v>
       </c>
     </row>
     <row r="282" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17094,10 +17423,10 @@
         <v>293</v>
       </c>
       <c r="B282" s="1">
-        <v>5.2632048700287699</v>
+        <v>5.2341542225512701</v>
       </c>
       <c r="C282" s="1">
-        <v>8.3922207540377103E-2</v>
+        <v>8.3819979532311101E-2</v>
       </c>
     </row>
     <row r="283" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17105,10 +17434,10 @@
         <v>294</v>
       </c>
       <c r="B283" s="1">
-        <v>5.2341542225512701</v>
+        <v>5.2499074678307798</v>
       </c>
       <c r="C283" s="1">
-        <v>8.3819979532311101E-2</v>
+        <v>8.4065913892834104E-2</v>
       </c>
     </row>
     <row r="284" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17116,10 +17445,10 @@
         <v>295</v>
       </c>
       <c r="B284" s="1">
-        <v>5.2499074678307798</v>
+        <v>5.2609478156281302</v>
       </c>
       <c r="C284" s="1">
-        <v>8.4065913892834104E-2</v>
+        <v>8.4094869806041694E-2</v>
       </c>
     </row>
     <row r="285" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17127,10 +17456,10 @@
         <v>296</v>
       </c>
       <c r="B285" s="1">
-        <v>5.2609478156281302</v>
+        <v>5.2522638411999596</v>
       </c>
       <c r="C285" s="1">
-        <v>8.4094869806041694E-2</v>
+        <v>8.3498425913598198E-2</v>
       </c>
     </row>
     <row r="286" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17138,10 +17467,10 @@
         <v>297</v>
       </c>
       <c r="B286" s="1">
-        <v>5.2522638411999596</v>
+        <v>5.2381148673874796</v>
       </c>
       <c r="C286" s="1">
-        <v>8.3498425913598198E-2</v>
+        <v>8.3501392552088799E-2</v>
       </c>
     </row>
     <row r="287" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17149,10 +17478,10 @@
         <v>298</v>
       </c>
       <c r="B287" s="1">
-        <v>5.2381148673874796</v>
+        <v>5.2236574261532196</v>
       </c>
       <c r="C287" s="1">
-        <v>8.3501392552088799E-2</v>
+        <v>8.3538886283743397E-2</v>
       </c>
     </row>
     <row r="288" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17160,10 +17489,10 @@
         <v>299</v>
       </c>
       <c r="B288" s="1">
-        <v>5.2236574261532196</v>
+        <v>5.2262449444555799</v>
       </c>
       <c r="C288" s="1">
-        <v>8.3538886283743397E-2</v>
+        <v>8.3653316711863296E-2</v>
       </c>
     </row>
     <row r="289" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17171,10 +17500,10 @@
         <v>300</v>
       </c>
       <c r="B289" s="1">
-        <v>5.2262449444555799</v>
+        <v>5.2457271314303799</v>
       </c>
       <c r="C289" s="1">
-        <v>8.3653316711863296E-2</v>
+        <v>8.36218907831483E-2</v>
       </c>
     </row>
     <row r="290" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17182,10 +17511,10 @@
         <v>301</v>
       </c>
       <c r="B290" s="1">
-        <v>5.2457271314303799</v>
+        <v>5.2597760818477397</v>
       </c>
       <c r="C290" s="1">
-        <v>8.36218907831483E-2</v>
+        <v>8.3768728051409405E-2</v>
       </c>
     </row>
     <row r="291" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17193,10 +17522,10 @@
         <v>302</v>
       </c>
       <c r="B291" s="1">
-        <v>5.2597760818477397</v>
+        <v>5.2273625593786797</v>
       </c>
       <c r="C291" s="1">
-        <v>8.3768728051409405E-2</v>
+        <v>8.3798815283381206E-2</v>
       </c>
     </row>
     <row r="292" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17204,10 +17533,10 @@
         <v>303</v>
       </c>
       <c r="B292" s="1">
-        <v>5.2273625593786797</v>
+        <v>5.2281725990355099</v>
       </c>
       <c r="C292" s="1">
-        <v>8.3798815283381206E-2</v>
+        <v>8.37952938220691E-2</v>
       </c>
     </row>
     <row r="293" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17215,10 +17544,10 @@
         <v>304</v>
       </c>
       <c r="B293" s="1">
-        <v>5.2281725990355099</v>
+        <v>5.2464873820867899</v>
       </c>
       <c r="C293" s="1">
-        <v>8.37952938220691E-2</v>
+        <v>8.4084000178888202E-2</v>
       </c>
     </row>
     <row r="294" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17226,10 +17555,10 @@
         <v>305</v>
       </c>
       <c r="B294" s="1">
-        <v>5.2464873820867899</v>
+        <v>5.2357499987829099</v>
       </c>
       <c r="C294" s="1">
-        <v>8.4084000178888202E-2</v>
+        <v>8.4478909636109295E-2</v>
       </c>
     </row>
     <row r="295" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17237,10 +17566,10 @@
         <v>306</v>
       </c>
       <c r="B295" s="1">
-        <v>5.2357499987829099</v>
+        <v>5.2426137496126399</v>
       </c>
       <c r="C295" s="1">
-        <v>8.4478909636109295E-2</v>
+        <v>8.4376066440544406E-2</v>
       </c>
     </row>
     <row r="296" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17248,10 +17577,10 @@
         <v>307</v>
       </c>
       <c r="B296" s="1">
-        <v>5.2426137496126399</v>
+        <v>5.25389374708476</v>
       </c>
       <c r="C296" s="1">
-        <v>8.4376066440544406E-2</v>
+        <v>8.42642456111901E-2</v>
       </c>
     </row>
     <row r="297" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17259,10 +17588,10 @@
         <v>308</v>
       </c>
       <c r="B297" s="1">
-        <v>5.25389374708476</v>
+        <v>5.2452132048918996</v>
       </c>
       <c r="C297" s="1">
-        <v>8.42642456111901E-2</v>
+        <v>8.3954508319290494E-2</v>
       </c>
     </row>
     <row r="298" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17270,10 +17599,10 @@
         <v>309</v>
       </c>
       <c r="B298" s="1">
-        <v>5.2452132048918996</v>
+        <v>5.2477036957110901</v>
       </c>
       <c r="C298" s="1">
-        <v>8.3954508319290494E-2</v>
+        <v>8.4241621326531999E-2</v>
       </c>
     </row>
     <row r="299" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17281,10 +17610,10 @@
         <v>310</v>
       </c>
       <c r="B299" s="1">
-        <v>5.2477036957110901</v>
+        <v>5.1912280334424699</v>
       </c>
       <c r="C299" s="1">
-        <v>8.4241621326531999E-2</v>
+        <v>8.39433811384213E-2</v>
       </c>
     </row>
     <row r="300" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17292,10 +17621,10 @@
         <v>311</v>
       </c>
       <c r="B300" s="1">
-        <v>5.1912280334424699</v>
+        <v>5.2649162726060403</v>
       </c>
       <c r="C300" s="1">
-        <v>8.39433811384213E-2</v>
+        <v>8.4883882170655206E-2</v>
       </c>
     </row>
     <row r="301" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17303,10 +17632,10 @@
         <v>312</v>
       </c>
       <c r="B301" s="1">
-        <v>5.2649162726060403</v>
+        <v>5.2682959002266401</v>
       </c>
       <c r="C301" s="1">
-        <v>8.4883882170655206E-2</v>
+        <v>8.4153042797615304E-2</v>
       </c>
     </row>
     <row r="302" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17314,10 +17643,10 @@
         <v>313</v>
       </c>
       <c r="B302" s="1">
-        <v>5.2682959002266401</v>
+        <v>4.0504847360743401</v>
       </c>
       <c r="C302" s="1">
-        <v>8.4153042797615304E-2</v>
+        <v>6.4664938143317294E-2</v>
       </c>
     </row>
     <row r="303" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17325,10 +17654,10 @@
         <v>314</v>
       </c>
       <c r="B303" s="1">
-        <v>4.0504847360743401</v>
+        <v>4.0496768121653703</v>
       </c>
       <c r="C303" s="1">
-        <v>6.4664938143317294E-2</v>
+        <v>6.48925563524336E-2</v>
       </c>
     </row>
     <row r="304" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17336,10 +17665,10 @@
         <v>315</v>
       </c>
       <c r="B304" s="1">
-        <v>4.0496768121653703</v>
+        <v>4.0401570007949097</v>
       </c>
       <c r="C304" s="1">
-        <v>6.48925563524336E-2</v>
+        <v>6.4717624366303003E-2</v>
       </c>
     </row>
     <row r="305" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17347,10 +17676,10 @@
         <v>316</v>
       </c>
       <c r="B305" s="1">
-        <v>4.0401570007949097</v>
+        <v>4.0452933053436704</v>
       </c>
       <c r="C305" s="1">
-        <v>6.4717624366303003E-2</v>
+        <v>6.5096945322289101E-2</v>
       </c>
     </row>
     <row r="306" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17358,10 +17687,10 @@
         <v>317</v>
       </c>
       <c r="B306" s="1">
-        <v>4.0452933053436704</v>
+        <v>4.0393053513377497</v>
       </c>
       <c r="C306" s="1">
-        <v>6.5096945322289101E-2</v>
+        <v>6.4780635694392893E-2</v>
       </c>
     </row>
     <row r="307" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17369,10 +17698,10 @@
         <v>318</v>
       </c>
       <c r="B307" s="1">
-        <v>4.0393053513377497</v>
+        <v>4.0427869051265404</v>
       </c>
       <c r="C307" s="1">
-        <v>6.4780635694392893E-2</v>
+        <v>6.4828747039054904E-2</v>
       </c>
     </row>
     <row r="308" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17380,10 +17709,10 @@
         <v>319</v>
       </c>
       <c r="B308" s="1">
-        <v>4.0427869051265404</v>
+        <v>4.0371132630075302</v>
       </c>
       <c r="C308" s="1">
-        <v>6.4828747039054904E-2</v>
+        <v>6.4845896931015903E-2</v>
       </c>
     </row>
     <row r="309" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17391,10 +17720,10 @@
         <v>320</v>
       </c>
       <c r="B309" s="1">
-        <v>4.0371132630075302</v>
+        <v>4.0301105995964903</v>
       </c>
       <c r="C309" s="1">
-        <v>6.4845896931015903E-2</v>
+        <v>6.4898532838035997E-2</v>
       </c>
     </row>
     <row r="310" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17402,10 +17731,10 @@
         <v>321</v>
       </c>
       <c r="B310" s="1">
-        <v>4.0301105995964903</v>
+        <v>4.0520999190004696</v>
       </c>
       <c r="C310" s="1">
-        <v>6.4898532838035997E-2</v>
+        <v>6.4393394651674596E-2</v>
       </c>
     </row>
     <row r="311" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17413,10 +17742,10 @@
         <v>322</v>
       </c>
       <c r="B311" s="1">
-        <v>4.0520999190004696</v>
+        <v>4.0532303423785203</v>
       </c>
       <c r="C311" s="1">
-        <v>6.4393394651674596E-2</v>
+        <v>6.4836933722996301E-2</v>
       </c>
     </row>
     <row r="312" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17424,10 +17753,10 @@
         <v>323</v>
       </c>
       <c r="B312" s="1">
-        <v>4.0532303423785203</v>
+        <v>4.0597656945719098</v>
       </c>
       <c r="C312" s="1">
-        <v>6.4836933722996301E-2</v>
+        <v>6.4898123293677099E-2</v>
       </c>
     </row>
     <row r="313" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17435,10 +17764,10 @@
         <v>324</v>
       </c>
       <c r="B313" s="1">
-        <v>4.0597656945719098</v>
+        <v>4.0397313521665303</v>
       </c>
       <c r="C313" s="1">
-        <v>6.4898123293677099E-2</v>
+        <v>6.48141939607636E-2</v>
       </c>
     </row>
     <row r="314" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17446,10 +17775,10 @@
         <v>325</v>
       </c>
       <c r="B314" s="1">
-        <v>4.0397313521665303</v>
+        <v>4.0389446603470498</v>
       </c>
       <c r="C314" s="1">
-        <v>6.48141939607636E-2</v>
+        <v>6.4945690313312696E-2</v>
       </c>
     </row>
     <row r="315" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17457,10 +17786,10 @@
         <v>326</v>
       </c>
       <c r="B315" s="1">
-        <v>4.0389446603470498</v>
+        <v>4.0491521884945199</v>
       </c>
       <c r="C315" s="1">
-        <v>6.4945690313312696E-2</v>
+        <v>6.4750632359324503E-2</v>
       </c>
     </row>
     <row r="316" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17468,10 +17797,10 @@
         <v>327</v>
       </c>
       <c r="B316" s="1">
-        <v>4.0491521884945199</v>
+        <v>4.0282207799584802</v>
       </c>
       <c r="C316" s="1">
-        <v>6.4750632359324503E-2</v>
+        <v>6.46466961945657E-2</v>
       </c>
     </row>
     <row r="317" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17479,10 +17808,10 @@
         <v>328</v>
       </c>
       <c r="B317" s="1">
-        <v>4.0282207799584802</v>
+        <v>4.0373666399902799</v>
       </c>
       <c r="C317" s="1">
-        <v>6.46466961945657E-2</v>
+        <v>6.5070391277710998E-2</v>
       </c>
     </row>
     <row r="318" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17490,10 +17819,10 @@
         <v>329</v>
       </c>
       <c r="B318" s="1">
-        <v>4.0373666399902799</v>
+        <v>4.0254616281370303</v>
       </c>
       <c r="C318" s="1">
-        <v>6.5070391277710998E-2</v>
+        <v>6.5003508402351404E-2</v>
       </c>
     </row>
     <row r="319" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17501,10 +17830,10 @@
         <v>330</v>
       </c>
       <c r="B319" s="1">
-        <v>4.0254616281370303</v>
+        <v>4.0346044905874798</v>
       </c>
       <c r="C319" s="1">
-        <v>6.5003508402351404E-2</v>
+        <v>6.4702157939462199E-2</v>
       </c>
     </row>
     <row r="320" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17512,10 +17841,10 @@
         <v>331</v>
       </c>
       <c r="B320" s="1">
-        <v>4.0346044905874798</v>
+        <v>4.0220126763814203</v>
       </c>
       <c r="C320" s="1">
-        <v>6.4702157939462199E-2</v>
+        <v>6.4789520162763903E-2</v>
       </c>
     </row>
     <row r="321" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17523,10 +17852,10 @@
         <v>332</v>
       </c>
       <c r="B321" s="1">
-        <v>4.0220126763814203</v>
+        <v>4.0377589881580498</v>
       </c>
       <c r="C321" s="1">
-        <v>6.4789520162763903E-2</v>
+        <v>6.4698100702121605E-2</v>
       </c>
     </row>
     <row r="322" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17534,10 +17863,10 @@
         <v>333</v>
       </c>
       <c r="B322" s="1">
-        <v>4.0377589881580498</v>
+        <v>4.0016969711271004</v>
       </c>
       <c r="C322" s="1">
-        <v>6.4698100702121605E-2</v>
+        <v>6.39060983563466E-2</v>
       </c>
     </row>
     <row r="323" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17545,10 +17874,10 @@
         <v>334</v>
       </c>
       <c r="B323" s="1">
-        <v>4.0016969711271004</v>
+        <v>3.9850777599500198</v>
       </c>
       <c r="C323" s="1">
-        <v>6.39060983563466E-2</v>
+        <v>6.4217223623450101E-2</v>
       </c>
     </row>
     <row r="324" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17556,10 +17885,10 @@
         <v>335</v>
       </c>
       <c r="B324" s="1">
-        <v>3.9850777599500198</v>
+        <v>4.0132441168710704</v>
       </c>
       <c r="C324" s="1">
-        <v>6.4217223623450101E-2</v>
+        <v>6.4146735969449406E-2</v>
       </c>
     </row>
     <row r="325" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17567,10 +17896,10 @@
         <v>336</v>
       </c>
       <c r="B325" s="1">
-        <v>4.0132441168710704</v>
+        <v>4.0107044449171996</v>
       </c>
       <c r="C325" s="1">
-        <v>6.4146735969449406E-2</v>
+        <v>6.4629796704458606E-2</v>
       </c>
     </row>
     <row r="326" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17578,10 +17907,10 @@
         <v>337</v>
       </c>
       <c r="B326" s="1">
-        <v>4.0107044449171996</v>
+        <v>4.0042080560711302</v>
       </c>
       <c r="C326" s="1">
-        <v>6.4629796704458606E-2</v>
+        <v>6.43943878164248E-2</v>
       </c>
     </row>
     <row r="327" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17589,10 +17918,10 @@
         <v>338</v>
       </c>
       <c r="B327" s="1">
-        <v>4.0042080560711302</v>
+        <v>4.0137738076926297</v>
       </c>
       <c r="C327" s="1">
-        <v>6.43943878164248E-2</v>
+        <v>6.4478725052475205E-2</v>
       </c>
     </row>
     <row r="328" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17600,10 +17929,10 @@
         <v>339</v>
       </c>
       <c r="B328" s="1">
-        <v>4.0137738076926297</v>
+        <v>4.0189067438591497</v>
       </c>
       <c r="C328" s="1">
-        <v>6.4478725052475205E-2</v>
+        <v>6.4781321835991806E-2</v>
       </c>
     </row>
     <row r="329" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17611,10 +17940,10 @@
         <v>340</v>
       </c>
       <c r="B329" s="1">
-        <v>4.0189067438591497</v>
+        <v>4.0019418304313801</v>
       </c>
       <c r="C329" s="1">
-        <v>6.4781321835991806E-2</v>
+        <v>6.4392626905219894E-2</v>
       </c>
     </row>
     <row r="330" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17622,10 +17951,10 @@
         <v>341</v>
       </c>
       <c r="B330" s="1">
-        <v>4.0019418304313801</v>
+        <v>4.0058057955871602</v>
       </c>
       <c r="C330" s="1">
-        <v>6.4392626905219894E-2</v>
+        <v>6.4250407980306304E-2</v>
       </c>
     </row>
     <row r="331" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17633,10 +17962,10 @@
         <v>342</v>
       </c>
       <c r="B331" s="1">
-        <v>4.0058057955871602</v>
+        <v>4.0060301681826802</v>
       </c>
       <c r="C331" s="1">
-        <v>6.4250407980306304E-2</v>
+        <v>6.4167196154649705E-2</v>
       </c>
     </row>
     <row r="332" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17644,10 +17973,10 @@
         <v>343</v>
       </c>
       <c r="B332" s="1">
-        <v>4.0060301681826802</v>
+        <v>3.99829105994908</v>
       </c>
       <c r="C332" s="1">
-        <v>6.4167196154649705E-2</v>
+        <v>6.4208136070914995E-2</v>
       </c>
     </row>
     <row r="333" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17655,10 +17984,10 @@
         <v>344</v>
       </c>
       <c r="B333" s="1">
-        <v>3.99829105994908</v>
+        <v>3.9906830558389799</v>
       </c>
       <c r="C333" s="1">
-        <v>6.4208136070914995E-2</v>
+        <v>6.4378306448205899E-2</v>
       </c>
     </row>
     <row r="334" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17666,10 +17995,10 @@
         <v>345</v>
       </c>
       <c r="B334" s="1">
-        <v>3.9906830558389799</v>
+        <v>3.99736506566357</v>
       </c>
       <c r="C334" s="1">
-        <v>6.4378306448205899E-2</v>
+        <v>6.4317608614747404E-2</v>
       </c>
     </row>
     <row r="335" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17677,10 +18006,10 @@
         <v>346</v>
       </c>
       <c r="B335" s="1">
-        <v>3.99736506566357</v>
+        <v>3.98390122498571</v>
       </c>
       <c r="C335" s="1">
-        <v>6.4317608614747404E-2</v>
+        <v>6.3677492575877404E-2</v>
       </c>
     </row>
     <row r="336" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17688,10 +18017,10 @@
         <v>347</v>
       </c>
       <c r="B336" s="1">
-        <v>3.98390122498571</v>
+        <v>3.9792620371784699</v>
       </c>
       <c r="C336" s="1">
-        <v>6.3677492575877404E-2</v>
+        <v>6.3641331008131394E-2</v>
       </c>
     </row>
     <row r="337" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17699,10 +18028,10 @@
         <v>348</v>
       </c>
       <c r="B337" s="1">
-        <v>3.9792620371784699</v>
+        <v>6.5540355078319896</v>
       </c>
       <c r="C337" s="1">
-        <v>6.3641331008131394E-2</v>
+        <v>0.105551348978041</v>
       </c>
     </row>
     <row r="338" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17710,10 +18039,10 @@
         <v>349</v>
       </c>
       <c r="B338" s="1">
-        <v>6.5540355078319896</v>
+        <v>6.5827244241657299</v>
       </c>
       <c r="C338" s="1">
-        <v>0.105551348978041</v>
+        <v>0.105991123494967</v>
       </c>
     </row>
     <row r="339" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17721,10 +18050,10 @@
         <v>350</v>
       </c>
       <c r="B339" s="1">
-        <v>6.5827244241657299</v>
+        <v>6.6067856280796899</v>
       </c>
       <c r="C339" s="1">
-        <v>0.105991123494967</v>
+        <v>0.10533604175596301</v>
       </c>
     </row>
     <row r="340" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17732,10 +18061,10 @@
         <v>351</v>
       </c>
       <c r="B340" s="1">
-        <v>6.6067856280796899</v>
+        <v>6.5726574723992401</v>
       </c>
       <c r="C340" s="1">
-        <v>0.10533604175596301</v>
+        <v>0.105665444142923</v>
       </c>
     </row>
     <row r="341" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17743,10 +18072,10 @@
         <v>352</v>
       </c>
       <c r="B341" s="1">
-        <v>6.5726574723992401</v>
+        <v>6.60849329589227</v>
       </c>
       <c r="C341" s="1">
-        <v>0.105665444142923</v>
+        <v>0.105198678205429</v>
       </c>
     </row>
     <row r="342" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17754,10 +18083,10 @@
         <v>353</v>
       </c>
       <c r="B342" s="1">
-        <v>6.60849329589227</v>
+        <v>6.61449436632694</v>
       </c>
       <c r="C342" s="1">
-        <v>0.105198678205429</v>
+        <v>0.105495395727284</v>
       </c>
     </row>
     <row r="343" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17765,10 +18094,10 @@
         <v>354</v>
       </c>
       <c r="B343" s="1">
-        <v>6.61449436632694</v>
+        <v>6.5773613187522404</v>
       </c>
       <c r="C343" s="1">
-        <v>0.105495395727284</v>
+        <v>0.105314548416934</v>
       </c>
     </row>
     <row r="344" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17776,10 +18105,10 @@
         <v>355</v>
       </c>
       <c r="B344" s="1">
-        <v>6.5773613187522404</v>
+        <v>6.6014893245484396</v>
       </c>
       <c r="C344" s="1">
-        <v>0.105314548416934</v>
+        <v>0.10568145895007799</v>
       </c>
     </row>
     <row r="345" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17787,10 +18116,10 @@
         <v>356</v>
       </c>
       <c r="B345" s="1">
-        <v>6.6014893245484396</v>
+        <v>6.5572879597699503</v>
       </c>
       <c r="C345" s="1">
-        <v>0.10568145895007799</v>
+        <v>0.10527614250211299</v>
       </c>
     </row>
     <row r="346" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17798,10 +18127,10 @@
         <v>357</v>
       </c>
       <c r="B346" s="1">
-        <v>6.5572879597699503</v>
+        <v>6.6008191975600301</v>
       </c>
       <c r="C346" s="1">
-        <v>0.10527614250211299</v>
+        <v>0.10576449952939899</v>
       </c>
     </row>
     <row r="347" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17809,10 +18138,10 @@
         <v>358</v>
       </c>
       <c r="B347" s="1">
-        <v>6.6008191975600301</v>
+        <v>6.6252507343515497</v>
       </c>
       <c r="C347" s="1">
-        <v>0.10576449952939899</v>
+        <v>0.10568293315542</v>
       </c>
     </row>
     <row r="348" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17820,10 +18149,10 @@
         <v>359</v>
       </c>
       <c r="B348" s="1">
-        <v>6.6252507343515497</v>
+        <v>6.5704906061544399</v>
       </c>
       <c r="C348" s="1">
-        <v>0.10568293315542</v>
+        <v>0.10581148690660699</v>
       </c>
     </row>
     <row r="349" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17831,10 +18160,10 @@
         <v>360</v>
       </c>
       <c r="B349" s="1">
-        <v>6.5704906061544399</v>
+        <v>6.5936568893976704</v>
       </c>
       <c r="C349" s="1">
-        <v>0.10581148690660699</v>
+        <v>0.105635832709833</v>
       </c>
     </row>
     <row r="350" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17842,10 +18171,10 @@
         <v>361</v>
       </c>
       <c r="B350" s="1">
-        <v>6.5936568893976704</v>
+        <v>6.5983973262679001</v>
       </c>
       <c r="C350" s="1">
-        <v>0.105635832709833</v>
+        <v>0.105645315996043</v>
       </c>
     </row>
     <row r="351" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17853,10 +18182,10 @@
         <v>362</v>
       </c>
       <c r="B351" s="1">
-        <v>6.5983973262679001</v>
+        <v>6.6115893763595901</v>
       </c>
       <c r="C351" s="1">
-        <v>0.105645315996043</v>
+        <v>0.105275447604903</v>
       </c>
     </row>
     <row r="352" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17864,10 +18193,10 @@
         <v>363</v>
       </c>
       <c r="B352" s="1">
-        <v>6.6115893763595901</v>
+        <v>6.5582265339750796</v>
       </c>
       <c r="C352" s="1">
-        <v>0.105275447604903</v>
+        <v>0.105662668847811</v>
       </c>
     </row>
     <row r="353" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17875,10 +18204,10 @@
         <v>364</v>
       </c>
       <c r="B353" s="1">
-        <v>6.5582265339750796</v>
+        <v>6.5712631537936099</v>
       </c>
       <c r="C353" s="1">
-        <v>0.105662668847811</v>
+        <v>0.105625257618033</v>
       </c>
     </row>
     <row r="354" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17886,10 +18215,10 @@
         <v>365</v>
       </c>
       <c r="B354" s="1">
-        <v>6.5712631537936099</v>
+        <v>6.6270719261065301</v>
       </c>
       <c r="C354" s="1">
-        <v>0.105625257618033</v>
+        <v>0.106115800022815</v>
       </c>
     </row>
     <row r="355" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17897,10 +18226,10 @@
         <v>366</v>
       </c>
       <c r="B355" s="1">
-        <v>6.6270719261065301</v>
+        <v>6.6192410240628501</v>
       </c>
       <c r="C355" s="1">
-        <v>0.106115800022815</v>
+        <v>0.106389444933465</v>
       </c>
     </row>
     <row r="356" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17908,10 +18237,10 @@
         <v>367</v>
       </c>
       <c r="B356" s="1">
-        <v>6.6192410240628501</v>
+        <v>6.57641937555222</v>
       </c>
       <c r="C356" s="1">
-        <v>0.106389444933465</v>
+        <v>0.105686237933491</v>
       </c>
     </row>
     <row r="357" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17919,10 +18248,10 @@
         <v>368</v>
       </c>
       <c r="B357" s="1">
-        <v>6.57641937555222</v>
+        <v>6.6087667968385899</v>
       </c>
       <c r="C357" s="1">
-        <v>0.105686237933491</v>
+        <v>0.106107125977925</v>
       </c>
     </row>
     <row r="358" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17930,10 +18259,10 @@
         <v>369</v>
       </c>
       <c r="B358" s="1">
-        <v>6.6087667968385899</v>
+        <v>6.5350348620169401</v>
       </c>
       <c r="C358" s="1">
-        <v>0.106107125977925</v>
+        <v>0.10569305527527301</v>
       </c>
     </row>
     <row r="359" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17941,10 +18270,10 @@
         <v>370</v>
       </c>
       <c r="B359" s="1">
-        <v>6.5350348620169401</v>
+        <v>6.5557760188699499</v>
       </c>
       <c r="C359" s="1">
-        <v>0.10569305527527301</v>
+        <v>0.105721916432143</v>
       </c>
     </row>
     <row r="360" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17952,10 +18281,10 @@
         <v>371</v>
       </c>
       <c r="B360" s="1">
-        <v>6.5557760188699499</v>
+        <v>5.9622611291336396</v>
       </c>
       <c r="C360" s="1">
-        <v>0.105721916432143</v>
+        <v>9.4951214409789694E-2</v>
       </c>
     </row>
     <row r="361" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17963,10 +18292,10 @@
         <v>372</v>
       </c>
       <c r="B361" s="1">
-        <v>6.5032195210687904</v>
+        <v>6.0066466306228703</v>
       </c>
       <c r="C361" s="1">
-        <v>0.10501733793063001</v>
+        <v>9.48427612752826E-2</v>
       </c>
     </row>
     <row r="362" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17974,10 +18303,10 @@
         <v>373</v>
       </c>
       <c r="B362" s="1">
-        <v>5.9622611291336396</v>
+        <v>5.9421219928096498</v>
       </c>
       <c r="C362" s="1">
-        <v>9.4951214409789694E-2</v>
+        <v>9.5323780436117694E-2</v>
       </c>
     </row>
     <row r="363" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17985,10 +18314,10 @@
         <v>374</v>
       </c>
       <c r="B363" s="1">
-        <v>6.0066466306228703</v>
+        <v>5.97435305885893</v>
       </c>
       <c r="C363" s="1">
-        <v>9.48427612752826E-2</v>
+        <v>9.5239680372887395E-2</v>
       </c>
     </row>
     <row r="364" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -17996,10 +18325,10 @@
         <v>375</v>
       </c>
       <c r="B364" s="1">
-        <v>5.9421219928096498</v>
+        <v>5.9503505932316996</v>
       </c>
       <c r="C364" s="1">
-        <v>9.5323780436117694E-2</v>
+        <v>9.4913957126963905E-2</v>
       </c>
     </row>
     <row r="365" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -18007,10 +18336,10 @@
         <v>376</v>
       </c>
       <c r="B365" s="1">
-        <v>5.97435305885893</v>
+        <v>5.9548297693894297</v>
       </c>
       <c r="C365" s="1">
-        <v>9.5239680372887395E-2</v>
+        <v>9.5207811574283305E-2</v>
       </c>
     </row>
     <row r="366" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -18018,10 +18347,10 @@
         <v>377</v>
       </c>
       <c r="B366" s="1">
-        <v>5.9503505932316996</v>
+        <v>5.9553030366034303</v>
       </c>
       <c r="C366" s="1">
-        <v>9.4913957126963905E-2</v>
+        <v>9.5333549341072299E-2</v>
       </c>
     </row>
     <row r="367" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -18029,10 +18358,10 @@
         <v>378</v>
       </c>
       <c r="B367" s="1">
-        <v>5.9548297693894297</v>
+        <v>5.9714415945772101</v>
       </c>
       <c r="C367" s="1">
-        <v>9.5207811574283305E-2</v>
+        <v>9.5272929905971096E-2</v>
       </c>
     </row>
     <row r="368" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -18040,10 +18369,10 @@
         <v>379</v>
       </c>
       <c r="B368" s="1">
-        <v>5.9553030366034303</v>
+        <v>5.9546595386126704</v>
       </c>
       <c r="C368" s="1">
-        <v>9.5333549341072299E-2</v>
+        <v>9.5825730092529093E-2</v>
       </c>
     </row>
     <row r="369" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -18051,10 +18380,10 @@
         <v>380</v>
       </c>
       <c r="B369" s="1">
-        <v>5.9714415945772101</v>
+        <v>5.9526717332290202</v>
       </c>
       <c r="C369" s="1">
-        <v>9.5272929905971096E-2</v>
+        <v>9.5557760398135405E-2</v>
       </c>
     </row>
     <row r="370" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -18062,10 +18391,10 @@
         <v>381</v>
       </c>
       <c r="B370" s="1">
-        <v>5.9546595386126704</v>
+        <v>5.9925762983853099</v>
       </c>
       <c r="C370" s="1">
-        <v>9.5825730092529093E-2</v>
+        <v>9.5707695616314301E-2</v>
       </c>
     </row>
     <row r="371" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -18073,10 +18402,10 @@
         <v>382</v>
       </c>
       <c r="B371" s="1">
-        <v>5.9526717332290202</v>
+        <v>5.9607737827043099</v>
       </c>
       <c r="C371" s="1">
-        <v>9.5557760398135405E-2</v>
+        <v>9.5513472864986904E-2</v>
       </c>
     </row>
     <row r="372" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -18084,10 +18413,10 @@
         <v>383</v>
       </c>
       <c r="B372" s="1">
-        <v>5.9925762983853099</v>
+        <v>5.9798136479539004</v>
       </c>
       <c r="C372" s="1">
-        <v>9.5707695616314301E-2</v>
+        <v>9.5307639125115001E-2</v>
       </c>
     </row>
     <row r="373" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -18095,10 +18424,10 @@
         <v>384</v>
       </c>
       <c r="B373" s="1">
-        <v>5.9607737827043099</v>
+        <v>5.9855117155737396</v>
       </c>
       <c r="C373" s="1">
-        <v>9.5513472864986904E-2</v>
+        <v>9.6102530139334702E-2</v>
       </c>
     </row>
     <row r="374" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -18106,10 +18435,10 @@
         <v>385</v>
       </c>
       <c r="B374" s="1">
-        <v>5.9798136479539004</v>
+        <v>6.0292733180363696</v>
       </c>
       <c r="C374" s="1">
-        <v>9.5307639125115001E-2</v>
+        <v>9.5842612321962603E-2</v>
       </c>
     </row>
     <row r="375" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -18117,10 +18446,10 @@
         <v>386</v>
       </c>
       <c r="B375" s="1">
-        <v>5.9855117155737396</v>
+        <v>5.9440797542562098</v>
       </c>
       <c r="C375" s="1">
-        <v>9.6102530139334702E-2</v>
+        <v>9.5502184039375396E-2</v>
       </c>
     </row>
     <row r="376" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -18128,10 +18457,10 @@
         <v>387</v>
       </c>
       <c r="B376" s="1">
-        <v>6.0292733180363696</v>
+        <v>5.9637069175640898</v>
       </c>
       <c r="C376" s="1">
-        <v>9.5842612321962603E-2</v>
+        <v>9.5885385701222001E-2</v>
       </c>
     </row>
     <row r="377" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -18139,10 +18468,10 @@
         <v>388</v>
       </c>
       <c r="B377" s="1">
-        <v>5.9440797542562098</v>
+        <v>5.9851248839214604</v>
       </c>
       <c r="C377" s="1">
-        <v>9.5502184039375396E-2</v>
+        <v>9.6439591076729503E-2</v>
       </c>
     </row>
     <row r="378" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -18150,10 +18479,10 @@
         <v>389</v>
       </c>
       <c r="B378" s="1">
-        <v>5.9637069175640898</v>
+        <v>5.9753311000708296</v>
       </c>
       <c r="C378" s="1">
-        <v>9.5885385701222001E-2</v>
+        <v>9.5315139971463694E-2</v>
       </c>
     </row>
     <row r="379" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -18161,10 +18490,10 @@
         <v>390</v>
       </c>
       <c r="B379" s="1">
-        <v>5.9851248839214604</v>
+        <v>5.95595351810669</v>
       </c>
       <c r="C379" s="1">
-        <v>9.6439591076729503E-2</v>
+        <v>9.5613752572800206E-2</v>
       </c>
     </row>
     <row r="380" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -18172,10 +18501,10 @@
         <v>391</v>
       </c>
       <c r="B380" s="1">
-        <v>5.9753311000708296</v>
+        <v>5.9436339167314696</v>
       </c>
       <c r="C380" s="1">
-        <v>9.5315139971463694E-2</v>
+        <v>9.57329103303277E-2</v>
       </c>
     </row>
     <row r="381" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -18183,10 +18512,10 @@
         <v>392</v>
       </c>
       <c r="B381" s="1">
-        <v>5.95595351810669</v>
+        <v>5.9680724903054401</v>
       </c>
       <c r="C381" s="1">
-        <v>9.5613752572800206E-2</v>
+        <v>9.4740461511437099E-2</v>
       </c>
     </row>
     <row r="382" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -18194,10 +18523,10 @@
         <v>393</v>
       </c>
       <c r="B382" s="1">
-        <v>5.9436339167314696</v>
+        <v>5.97890051441588</v>
       </c>
       <c r="C382" s="1">
-        <v>9.57329103303277E-2</v>
+        <v>9.56068005906138E-2</v>
       </c>
     </row>
     <row r="383" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -18205,10 +18534,10 @@
         <v>394</v>
       </c>
       <c r="B383" s="1">
-        <v>5.9680724903054401</v>
+        <v>5.9641145262355701</v>
       </c>
       <c r="C383" s="1">
-        <v>9.4740461511437099E-2</v>
+        <v>9.5241121615471297E-2</v>
       </c>
     </row>
     <row r="384" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -18216,10 +18545,10 @@
         <v>395</v>
       </c>
       <c r="B384" s="1">
-        <v>5.97890051441588</v>
+        <v>5.9548137587277301</v>
       </c>
       <c r="C384" s="1">
-        <v>9.56068005906138E-2</v>
+        <v>9.5433597155929403E-2</v>
       </c>
     </row>
     <row r="385" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -18227,10 +18556,10 @@
         <v>396</v>
       </c>
       <c r="B385" s="1">
-        <v>5.9641145262355701</v>
+        <v>5.9412161279185698</v>
       </c>
       <c r="C385" s="1">
-        <v>9.5241121615471297E-2</v>
+        <v>9.5987289369727502E-2</v>
       </c>
     </row>
     <row r="386" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -18238,10 +18567,10 @@
         <v>397</v>
       </c>
       <c r="B386" s="1">
-        <v>5.9548137587277301</v>
+        <v>5.9237749973025897</v>
       </c>
       <c r="C386" s="1">
-        <v>9.5433597155929403E-2</v>
+        <v>9.5313166809118E-2</v>
       </c>
     </row>
     <row r="387" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -18249,10 +18578,10 @@
         <v>398</v>
       </c>
       <c r="B387" s="1">
-        <v>5.9412161279185698</v>
+        <v>5.9321677454244002</v>
       </c>
       <c r="C387" s="1">
-        <v>9.5987289369727502E-2</v>
+        <v>9.5108590519696196E-2</v>
       </c>
     </row>
     <row r="388" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -18260,10 +18589,10 @@
         <v>399</v>
       </c>
       <c r="B388" s="1">
-        <v>5.9237749973025897</v>
+        <v>5.9655682681986404</v>
       </c>
       <c r="C388" s="1">
-        <v>9.5313166809118E-2</v>
+        <v>9.5279653817559096E-2</v>
       </c>
     </row>
     <row r="389" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -18271,10 +18600,10 @@
         <v>400</v>
       </c>
       <c r="B389" s="1">
-        <v>5.9321677454244002</v>
+        <v>5.9648566611082501</v>
       </c>
       <c r="C389" s="1">
-        <v>9.5108590519696196E-2</v>
+        <v>9.5070431421425905E-2</v>
       </c>
     </row>
     <row r="390" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -18282,10 +18611,10 @@
         <v>401</v>
       </c>
       <c r="B390" s="1">
-        <v>5.9655682681986404</v>
+        <v>3.0672817324059798</v>
       </c>
       <c r="C390" s="1">
-        <v>9.5279653817559096E-2</v>
+        <v>4.9220544832568401E-2</v>
       </c>
     </row>
     <row r="391" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -18293,10 +18622,340 @@
         <v>402</v>
       </c>
       <c r="B391" s="1">
-        <v>5.9648566611082501</v>
+        <v>3.06498328697809</v>
       </c>
       <c r="C391" s="1">
-        <v>9.5070431421425905E-2</v>
+        <v>4.8826525513616603E-2</v>
+      </c>
+    </row>
+    <row r="392" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A392" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="B392" s="1">
+        <v>3.06753441554193</v>
+      </c>
+      <c r="C392" s="1">
+        <v>4.9256122272570202E-2</v>
+      </c>
+    </row>
+    <row r="393" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A393" s="1" t="s">
+        <v>404</v>
+      </c>
+      <c r="B393" s="1">
+        <v>3.0756019900176499</v>
+      </c>
+      <c r="C393" s="1">
+        <v>4.97179954883646E-2</v>
+      </c>
+    </row>
+    <row r="394" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A394" s="1" t="s">
+        <v>405</v>
+      </c>
+      <c r="B394" s="1">
+        <v>3.0649036050172098</v>
+      </c>
+      <c r="C394" s="1">
+        <v>4.9725118840505199E-2</v>
+      </c>
+    </row>
+    <row r="395" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A395" s="1" t="s">
+        <v>406</v>
+      </c>
+      <c r="B395" s="1">
+        <v>3.06529341587372</v>
+      </c>
+      <c r="C395" s="1">
+        <v>4.9381962862556E-2</v>
+      </c>
+    </row>
+    <row r="396" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A396" s="1" t="s">
+        <v>407</v>
+      </c>
+      <c r="B396" s="1">
+        <v>3.0726606549971298</v>
+      </c>
+      <c r="C396" s="1">
+        <v>4.8979944321647401E-2</v>
+      </c>
+    </row>
+    <row r="397" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A397" s="1" t="s">
+        <v>408</v>
+      </c>
+      <c r="B397" s="1">
+        <v>3.0831176610414701</v>
+      </c>
+      <c r="C397" s="1">
+        <v>4.9045485231240298E-2</v>
+      </c>
+    </row>
+    <row r="398" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A398" s="1" t="s">
+        <v>409</v>
+      </c>
+      <c r="B398" s="1">
+        <v>3.0668965665752701</v>
+      </c>
+      <c r="C398" s="1">
+        <v>4.8965298287210399E-2</v>
+      </c>
+    </row>
+    <row r="399" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A399" s="1" t="s">
+        <v>410</v>
+      </c>
+      <c r="B399" s="1">
+        <v>3.0577539539137901</v>
+      </c>
+      <c r="C399" s="1">
+        <v>4.8957627310304702E-2</v>
+      </c>
+    </row>
+    <row r="400" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A400" s="1" t="s">
+        <v>411</v>
+      </c>
+      <c r="B400" s="1">
+        <v>3.0461287705788598</v>
+      </c>
+      <c r="C400" s="1">
+        <v>4.9000057015244597E-2</v>
+      </c>
+    </row>
+    <row r="401" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A401" s="1" t="s">
+        <v>412</v>
+      </c>
+      <c r="B401" s="1">
+        <v>3.0420177016521102</v>
+      </c>
+      <c r="C401" s="1">
+        <v>4.8651617087087401E-2</v>
+      </c>
+    </row>
+    <row r="402" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A402" s="1" t="s">
+        <v>413</v>
+      </c>
+      <c r="B402" s="1">
+        <v>3.0577648925430601</v>
+      </c>
+      <c r="C402" s="1">
+        <v>4.8810930819998197E-2</v>
+      </c>
+    </row>
+    <row r="403" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A403" s="1" t="s">
+        <v>414</v>
+      </c>
+      <c r="B403" s="1">
+        <v>3.07207699092403</v>
+      </c>
+      <c r="C403" s="1">
+        <v>4.8901071369119802E-2</v>
+      </c>
+    </row>
+    <row r="404" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A404" s="1" t="s">
+        <v>415</v>
+      </c>
+      <c r="B404" s="1">
+        <v>3.0603120961688499</v>
+      </c>
+      <c r="C404" s="1">
+        <v>4.9126205451321202E-2</v>
+      </c>
+    </row>
+    <row r="405" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A405" s="1" t="s">
+        <v>416</v>
+      </c>
+      <c r="B405" s="1">
+        <v>3.0495273783215602</v>
+      </c>
+      <c r="C405" s="1">
+        <v>4.95058693259324E-2</v>
+      </c>
+    </row>
+    <row r="406" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A406" s="1" t="s">
+        <v>417</v>
+      </c>
+      <c r="B406" s="1">
+        <v>3.0483213432966099</v>
+      </c>
+      <c r="C406" s="1">
+        <v>4.8651769164606402E-2</v>
+      </c>
+    </row>
+    <row r="407" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A407" s="1" t="s">
+        <v>418</v>
+      </c>
+      <c r="B407" s="1">
+        <v>3.0507028081060601</v>
+      </c>
+      <c r="C407" s="1">
+        <v>4.8908241247632697E-2</v>
+      </c>
+    </row>
+    <row r="408" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A408" s="1" t="s">
+        <v>419</v>
+      </c>
+      <c r="B408" s="1">
+        <v>3.0503873160495498</v>
+      </c>
+      <c r="C408" s="1">
+        <v>4.8699146330509702E-2</v>
+      </c>
+    </row>
+    <row r="409" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A409" s="1" t="s">
+        <v>420</v>
+      </c>
+      <c r="B409" s="1">
+        <v>3.0616213771126799</v>
+      </c>
+      <c r="C409" s="1">
+        <v>4.91555175312548E-2</v>
+      </c>
+    </row>
+    <row r="410" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A410" s="1" t="s">
+        <v>421</v>
+      </c>
+      <c r="B410" s="1">
+        <v>3.0441812745358798</v>
+      </c>
+      <c r="C410" s="1">
+        <v>4.9268660787059597E-2</v>
+      </c>
+    </row>
+    <row r="411" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A411" s="1" t="s">
+        <v>422</v>
+      </c>
+      <c r="B411" s="1">
+        <v>3.0545733491419398</v>
+      </c>
+      <c r="C411" s="1">
+        <v>4.8826826414769098E-2</v>
+      </c>
+    </row>
+    <row r="412" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A412" s="1" t="s">
+        <v>423</v>
+      </c>
+      <c r="B412" s="1">
+        <v>3.0565111313221198</v>
+      </c>
+      <c r="C412" s="1">
+        <v>4.8764627198113697E-2</v>
+      </c>
+    </row>
+    <row r="413" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A413" s="1" t="s">
+        <v>424</v>
+      </c>
+      <c r="B413" s="1">
+        <v>3.0569612836170998</v>
+      </c>
+      <c r="C413" s="1">
+        <v>4.9029160899217702E-2</v>
+      </c>
+    </row>
+    <row r="414" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A414" s="1" t="s">
+        <v>425</v>
+      </c>
+      <c r="B414" s="1">
+        <v>3.0531280697850698</v>
+      </c>
+      <c r="C414" s="1">
+        <v>4.8854122518207498E-2</v>
+      </c>
+    </row>
+    <row r="415" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A415" s="1" t="s">
+        <v>426</v>
+      </c>
+      <c r="B415" s="1">
+        <v>3.0495276887412501</v>
+      </c>
+      <c r="C415" s="1">
+        <v>4.9133881801381701E-2</v>
+      </c>
+    </row>
+    <row r="416" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A416" s="1" t="s">
+        <v>427</v>
+      </c>
+      <c r="B416" s="1">
+        <v>3.0451824247254602</v>
+      </c>
+      <c r="C416" s="1">
+        <v>4.9071806924917999E-2</v>
+      </c>
+    </row>
+    <row r="417" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A417" s="1" t="s">
+        <v>428</v>
+      </c>
+      <c r="B417" s="1">
+        <v>3.0636069285517098</v>
+      </c>
+      <c r="C417" s="1">
+        <v>4.9142870700877098E-2</v>
+      </c>
+    </row>
+    <row r="418" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A418" s="1" t="s">
+        <v>429</v>
+      </c>
+      <c r="B418" s="1">
+        <v>3.0573709331599099</v>
+      </c>
+      <c r="C418" s="1">
+        <v>4.9249210174874901E-2</v>
+      </c>
+    </row>
+    <row r="419" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A419" s="1" t="s">
+        <v>430</v>
+      </c>
+      <c r="B419" s="1">
+        <v>3.0482345249944598</v>
+      </c>
+      <c r="C419" s="1">
+        <v>4.8951873888496603E-2</v>
+      </c>
+    </row>
+    <row r="420" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A420" s="1" t="s">
+        <v>431</v>
+      </c>
+      <c r="B420" s="1">
+        <v>3.0486121479316401</v>
+      </c>
+      <c r="C420" s="1">
+        <v>4.8933368456572202E-2</v>
+      </c>
+    </row>
+    <row r="421" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A421" s="1" t="s">
+        <v>432</v>
+      </c>
+      <c r="B421" s="1">
+        <v>3.0547580292283598</v>
+      </c>
+      <c r="C421" s="1">
+        <v>4.87619094275357E-2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>